<commit_message>
fix: nomes neutros para efeitos genericos e linha 'Na Pokedex' em cada habilidade
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/habilidades-passivas-mascotes.xlsx
+++ b/docs/habilidades-passivas-mascotes.xlsx
@@ -660,7 +660,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Poder bruto</t>
+          <t>Ataque reforçado</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1398,7 +1398,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1603,7 +1603,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Casco</t>
+          <t>Defesa leve</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2373,7 +2373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N307"/>
+  <dimension ref="A1:O307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2390,6 +2390,7 @@
     <col width="8" customWidth="1" min="12" max="12"/>
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="60" customWidth="1" min="14" max="14"/>
+    <col width="60" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2463,6 +2464,11 @@
           <t>Original (Pokédex, inglês)</t>
         </is>
       </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Na Pokédex (resumo)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2522,6 +2528,11 @@
           <t>Increases the same-type attack bonus from 1.5× to 2×.</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>O bônus de mesmo tipo (STAB) passa de 1,5× para 2×.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2586,6 +2597,11 @@
           <t>Turns the bearer's Normal moves into Flying moves and strengthens them to 1.3× their power.</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Golpes Normais viram Voadores, mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2645,6 +2661,11 @@
           <t>Damages the attacker for 1/4 its max HP when knocked out by a contact move.</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Machuca quem o derrota com contato.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2734,6 +2755,11 @@
           <t>Strengthens moves to 1.3× their power when moving last.</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Golpes mais fortes se agir por último.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2793,6 +2819,11 @@
           <t>Raises Attack to the maximum of six stages upon receiving a critical hit.</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Ataque vai ao máximo ao receber um golpe crítico.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2852,6 +2883,11 @@
           <t>When the Pokémon's HP drops below half, Anger Shell lowers its Defense and Special Defense but its Attack, Special Attack and Speed are raised.</t>
         </is>
       </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Com HP abaixo da metade, ganha ataque e perde defesa.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2976,6 +3012,11 @@
           <t>Prevents the opponent from using any moves that have priority, such as Quick Attack.</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Impede os rivais de usar golpes com prioridade.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3035,6 +3076,11 @@
           <t>Protects allies against moves that affect their mental state.</t>
         </is>
       </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Protege aliados de efeitos que afetam a mente.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3094,6 +3140,11 @@
           <t>Combines the effects of Unnerve and Chilling Neigh.</t>
         </is>
       </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Combina Unnerve (impede frutas) e Chilling Neigh (Ataque sobe ao derrotar).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3153,6 +3204,11 @@
           <t>Combines the effects of Unnerve and Grim Neigh.</t>
         </is>
       </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Combina Unnerve (impede frutas) e Grim Neigh (Ataque Especial sobe ao derrotar).</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3202,7 +3258,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Casco</t>
+          <t>Defesa leve</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -3242,6 +3298,11 @@
           <t>A Pokémon with Aura Guard takes half damage from moves that make contact.</t>
         </is>
       </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Reduz pela metade o dano de golpes de contato.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -3361,6 +3422,11 @@
           <t>Ally Pokémon's moves have their power increased to 1.3×.</t>
         </is>
       </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Aumenta o poder dos golpes especiais dos aliados.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -3380,7 +3446,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Casco</t>
+          <t>Defesa leve</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -3420,6 +3486,11 @@
           <t>Protects against critical hits.</t>
         </is>
       </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Impede golpes críticos.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -3479,6 +3550,11 @@
           <t>Transforms this Pokémon into Ash-Greninja after fainting an opponent.  Water Shuriken's power is 20 and always hits three times.</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Transforma-se ao derrotar um Pokémon.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3543,6 +3619,11 @@
           <t>Lowers Special Defense of all Pokémon except itself.</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Reduz a Defesa Especial de todos os outros Pokémon.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3602,6 +3683,11 @@
           <t>Raises this Pokémon's highest stat by one stage when it faints another Pokémon.</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>O maior atributo sobe ao derrotar um Pokémon.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3661,6 +3747,11 @@
           <t>Raises this Pokémon's Special Attack by one stage every time its HP drops below half.</t>
         </is>
       </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Ataque Especial sobe quando o HP cai abaixo da metade.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3680,7 +3771,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3720,6 +3811,11 @@
           <t>Protects against Defense drops.</t>
         </is>
       </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>Impede que a Defesa seja reduzida.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3784,6 +3880,11 @@
           <t>Strengthens Fire moves to inflict 1.5× damage at 1/3 max HP or less.</t>
         </is>
       </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>Golpes de Fogo ficam mais fortes com HP baixo.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3803,7 +3904,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Casco</t>
+          <t>Defesa leve</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3843,6 +3944,11 @@
           <t>Protects against bullet, ball, and bomb-based moves.</t>
         </is>
       </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>Bloqueia golpes de bomba, bola e projétil.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3902,6 +4008,11 @@
           <t>Restores HP upon eating a Berry, in addition to the Berry's effect.</t>
         </is>
       </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>Recupera HP ao comer uma fruta.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3961,6 +4072,11 @@
           <t>Boosts Attack after knocking out a Pokémon.</t>
         </is>
       </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>Ataque sobe ao derrotar um Pokémon.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4020,6 +4136,11 @@
           <t>Doubles Speed during strong sunlight.</t>
         </is>
       </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>Dobra a Velocidade sob sol forte.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4039,7 +4160,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -4079,6 +4200,11 @@
           <t>Prevents stats from being lowered by other Pokémon.</t>
         </is>
       </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>Impede que outros Pokémon reduzam seus atributos.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -4258,6 +4384,11 @@
           <t>Raises Special Attack by two stages upon having any stat lowered.</t>
         </is>
       </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>Ataque Especial sobe muito ao ter um atributo reduzido.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4277,7 +4408,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -4317,6 +4448,11 @@
           <t>Increases moves' accuracy to 1.3×.</t>
         </is>
       </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>Aumenta a precisão dos golpes.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4411,6 +4547,11 @@
           <t>This Pokémon can inflict poison on Poison and Steel Pokémon.</t>
         </is>
       </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>Pode envenenar Pokémon de Aço e Veneno.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4470,6 +4611,11 @@
           <t>Copies ally's stat changes on entering battle.</t>
         </is>
       </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>Copia as mudanças de atributo de um aliado ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4534,6 +4680,11 @@
           <t>When Ignores moves and abilities that draw in moves.</t>
         </is>
       </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>Reduz a Velocidade de todos quando atingido.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4593,6 +4744,11 @@
           <t>Causes the Pokémon to reuse an already consumed Berry at the end of the next turn.</t>
         </is>
       </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>Reaproveita uma fruta já comida.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4657,6 +4813,11 @@
           <t>Has a 30% chance of Disabling any move that hits the Pokémon.</t>
         </is>
       </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>30% de chance de bloquear o golpe que o atingiu.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4721,6 +4882,11 @@
           <t>Has a 30% chance of infatuating attacking Pokémon on contact.</t>
         </is>
       </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>30% de chance de causar paixão em quem faz contato.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4845,6 +5011,11 @@
           <t>Strengthens Dark moves to 1.33× their power for all friendly and opposing Pokémon.</t>
         </is>
       </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>Golpes Sombrios de todos ficam mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4904,6 +5075,11 @@
           <t>Boosts Defense in battle.</t>
         </is>
       </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>Aumenta a Defesa ao entrar em combate.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4968,6 +5144,11 @@
           <t>Opposing Pokémon cannot use priority attacks.</t>
         </is>
       </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>Impede os rivais de usar golpes com prioridade.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5057,6 +5238,11 @@
           <t>Raises Attack two stages upon having any stat lowered.</t>
         </is>
       </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>Ataque sobe muito ao ter um atributo reduzido.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5121,6 +5307,11 @@
           <t>Creates a mysterious air current, which cannot be replaced and causes moves to never be super effective against Flying Pokémon.</t>
         </is>
       </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>Cria uma corrente que anula as fraquezas dos Voadores.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -5185,6 +5376,11 @@
           <t>Creates extremely harsh sunlight, which has all the properties of Sunny Day, cannot be replaced, and causes damaging Water moves to fail.</t>
         </is>
       </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>Invoca sol extremo ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -5244,6 +5440,11 @@
           <t>Prevents the first instance of battle damage.</t>
         </is>
       </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>Um disfarce absorve o primeiro golpe.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -5303,6 +5504,11 @@
           <t>Raises the attack stat corresponding to the opponents' weaker defense one stage upon entering battle.</t>
         </is>
       </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>Aumenta o ataque que explora a defesa mais fraca do rival.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5367,6 +5573,11 @@
           <t>The Pokémon's Normal-type moves become Dragon-type moves and their power is boosted by 20%.</t>
         </is>
       </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>Golpes Normais viram Dragão, mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5431,6 +5642,11 @@
           <t>Powers up Dragon-type moves.</t>
         </is>
       </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>Golpes de Dragão ficam mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5495,6 +5711,11 @@
           <t>Summons rain that lasts indefinitely upon entering battle.</t>
         </is>
       </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>Invoca chuva ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5559,6 +5780,11 @@
           <t>Summons strong sunlight that lasts indefinitely upon entering battle.</t>
         </is>
       </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>Invoca sol forte ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5618,6 +5844,11 @@
           <t>Causes 1/8 max HP in damage each turn during strong sunlight, but heals for 1/8 max HP during rain.  Increases damage from Fire moves to 1.25×, but absorbs Water moves, healing for 1/4 max HP.</t>
         </is>
       </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>Recupera HP na chuva e perde sob sol forte.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5712,6 +5943,11 @@
           <t>Restores HP when hit by a Ground-type move.</t>
         </is>
       </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>Recupera HP ao ser atingido por golpes de Terra.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5776,6 +6012,11 @@
           <t>The Pokémon floats off the ground, making it immune to Ground-type moves, as well as the Spikes, Toxic Spikes, and Sticky Web statuses. When the Pokémon knocks out a target with an attack, its highest stat is boosted by 1 stage.</t>
         </is>
       </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>Flutua: imune a golpes de Terra.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5840,6 +6081,11 @@
           <t>Has a 30% chance of inflcting either paralysis, poison, or sleep on attacking Pokémon on contact.</t>
         </is>
       </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>30% de chance de causar paralisia, veneno ou sono em quem faz contato.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5904,6 +6150,11 @@
           <t>When this Pokémon enters battle, it changes the terrain to Electric Terrain.</t>
         </is>
       </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>Cria terreno elétrico ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5963,6 +6214,11 @@
           <t>When hit by an attack, the power of the next Electric-type move it uses is doubled.</t>
         </is>
       </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>Ao ser atingido, o próximo golpe Elétrico dobra de poder.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -6022,6 +6278,11 @@
           <t>This Pokémon automatically switches out when its HP drops below half.</t>
         </is>
       </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>Sai de campo quando o HP cai abaixo da metade.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -6086,6 +6347,11 @@
           <t>Strengthens Fairy moves to 1.33× their power for all friendly and opposing Pokémon.</t>
         </is>
       </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>Golpes de Fada de todos ficam mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -6145,6 +6411,11 @@
           <t>Decreases damage taken from super-effective moves by 1/4.</t>
         </is>
       </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>Reduz o dano de golpes super efetivos.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -6209,6 +6480,11 @@
           <t>Boosts the power of the Pokémon's Fire-type moves by 50%.</t>
         </is>
       </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>Golpes de Fogo ficam mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -6273,6 +6549,11 @@
           <t>Has a 30% chance of burning attacking Pokémon on contact.</t>
         </is>
       </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>30% de chance de queimar quem faz contato.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -6332,6 +6613,11 @@
           <t>Increases Special Attack to 1.5× when burned.</t>
         </is>
       </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>Ataque Especial maior quando queimado.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6396,6 +6682,11 @@
           <t>Protects against Fire moves.  Once one has been blocked, the Pokémon's own Fire moves inflict 1.5× damage until it leaves battle.</t>
         </is>
       </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>Imune a Fogo e, ao absorver, fortalece os próprios golpes de Fogo.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6455,6 +6746,11 @@
           <t>Increases friendly Pokémon's Attack and Special Defense to 1.5× during strong sunlight.</t>
         </is>
       </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>Aumenta Ataque e Defesa Especial dos aliados sob sol forte.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6514,6 +6810,11 @@
           <t>Protects friendly Grass Pokémon from having their stats lowered by other Pokémon.</t>
         </is>
       </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>Protege aliados de Planta de perder atributos.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6533,7 +6834,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Casco</t>
+          <t>Defesa leve</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -6573,6 +6874,11 @@
           <t>Damage from contact moves is halved.  Damage from Fire moves is doubled.</t>
         </is>
       </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>Reduz pela metade o dano de contato (mas dobra o de Fogo).</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6692,6 +6998,11 @@
           <t>Decreases all direct damage taken by friendly Pokémon to 0.75×.</t>
         </is>
       </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>Reduz o dano que os aliados recebem.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6741,7 +7052,7 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -6781,6 +7092,11 @@
           <t>Other Pokémon cannot lower this Pokémon's stats.</t>
         </is>
       </c>
+      <c r="O81" t="inlineStr">
+        <is>
+          <t>Impede que outros Pokémon reduzam seus atributos.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6800,7 +7116,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Casco</t>
+          <t>Defesa leve</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -6840,6 +7156,11 @@
           <t>Halves damage from physical attacks.</t>
         </is>
       </c>
+      <c r="O82" t="inlineStr">
+        <is>
+          <t>Reduz pela metade o dano físico.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6899,6 +7220,11 @@
           <t>Raises Flying moves' priority by one stage.</t>
         </is>
       </c>
+      <c r="O83" t="inlineStr">
+        <is>
+          <t>Golpes Voadores agem primeiro.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6948,7 +7274,7 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -6988,6 +7314,11 @@
           <t>Gives immunity to status moves.</t>
         </is>
       </c>
+      <c r="O85" t="inlineStr">
+        <is>
+          <t>Imune a golpes de status.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7052,6 +7383,11 @@
           <t>Lowers attacking Pokémon's Speed by one stage on contact.</t>
         </is>
       </c>
+      <c r="O86" t="inlineStr">
+        <is>
+          <t>Reduz a Velocidade de quem faz contato.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7071,7 +7407,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Poder bruto</t>
+          <t>Ataque reforçado</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -7111,6 +7447,11 @@
           <t>Boosts the Pokémon's Attack stat but only allows the use of the first selected move.</t>
         </is>
       </c>
+      <c r="O87" t="inlineStr">
+        <is>
+          <t>Ataque maior, mas fica preso ao primeiro golpe escolhido.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7170,6 +7511,11 @@
           <t>Boosts Defense while Grassy Terrain is in effect.</t>
         </is>
       </c>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>Aumenta a Defesa em terreno de grama.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7234,6 +7580,11 @@
           <t>When this Pokémon enters battle, it changes the terrain to Grassy Terrain.</t>
         </is>
       </c>
+      <c r="O89" t="inlineStr">
+        <is>
+          <t>Cria terreno de grama ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7293,6 +7644,11 @@
           <t>Boosts Special Attack after knocking out a Pokémon.</t>
         </is>
       </c>
+      <c r="O90" t="inlineStr">
+        <is>
+          <t>Ataque Especial sobe ao derrotar um Pokémon.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7352,6 +7708,11 @@
           <t>Boosts Attack if intimidated, and prevents being forced to switch out.</t>
         </is>
       </c>
+      <c r="O91" t="inlineStr">
+        <is>
+          <t>Ataque sobe se for intimidado.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7441,6 +7802,11 @@
           <t>Increases Attack to 1.5× with a major status ailment.</t>
         </is>
       </c>
+      <c r="O93" t="inlineStr">
+        <is>
+          <t>Ataque maior quando está com problema de status.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7505,6 +7871,11 @@
           <t>Creates an Electric Terrain when entering battle, and boosts Special Attack while active.</t>
         </is>
       </c>
+      <c r="O94" t="inlineStr">
+        <is>
+          <t>Cria terreno elétrico e aumenta o Ataque Especial.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7564,6 +7935,11 @@
           <t>Has a 50% chance of restoring a used Berry after each turn if the Pokémon has held no items in the meantime.</t>
         </is>
       </c>
+      <c r="O95" t="inlineStr">
+        <is>
+          <t>Pode recuperar a fruta usada.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7623,6 +7999,11 @@
           <t>Has a 30% chance of curing each adjacent ally of any major status ailment after each turn.</t>
         </is>
       </c>
+      <c r="O96" t="inlineStr">
+        <is>
+          <t>Chance de curar o status de aliados todo turno.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7687,6 +8068,11 @@
           <t>Halves damage from Fire moves and burns.</t>
         </is>
       </c>
+      <c r="O97" t="inlineStr">
+        <is>
+          <t>Reduz pela metade o dano de Fogo e queimaduras.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -7806,6 +8192,11 @@
           <t>When a Pokémon with Hospitality enters a battle, it restores HP for an ally by 25%.</t>
         </is>
       </c>
+      <c r="O100" t="inlineStr">
+        <is>
+          <t>Ao entrar, recupera HP de um aliado.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -7825,7 +8216,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Poder bruto</t>
+          <t>Ataque reforçado</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -7865,6 +8256,11 @@
           <t>Doubles Attack in battle.</t>
         </is>
       </c>
+      <c r="O101" t="inlineStr">
+        <is>
+          <t>Dobra o Ataque.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -7914,7 +8310,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Poder bruto</t>
+          <t>Ataque reforçado</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -7954,6 +8350,11 @@
           <t>Strengthens physical moves to inflict 1.5× damage, but decreases their accuracy to 0.8×.</t>
         </is>
       </c>
+      <c r="O103" t="inlineStr">
+        <is>
+          <t>Golpes físicos mais fortes, porém menos precisos.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -8013,6 +8414,11 @@
           <t>Cures any major status ailment after each turn during rain.</t>
         </is>
       </c>
+      <c r="O104" t="inlineStr">
+        <is>
+          <t>Cura status todo turno na chuva.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -8032,7 +8438,7 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -8072,6 +8478,11 @@
           <t>Prevents Attack from being lowered by other Pokémon.</t>
         </is>
       </c>
+      <c r="O105" t="inlineStr">
+        <is>
+          <t>Impede que o Ataque seja reduzido.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -8131,6 +8542,11 @@
           <t>Heals for 1/16 max HP after each turn during hail.  Protects against hail damage.</t>
         </is>
       </c>
+      <c r="O106" t="inlineStr">
+        <is>
+          <t>Recupera um pouco de HP todo turno no granizo.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -8190,6 +8606,11 @@
           <t>The Pokémon’s ice head can take a physical attack as a substitute, but the attack also changes the Pokémon’s appearance. The ice will be restored when it snows.</t>
         </is>
       </c>
+      <c r="O107" t="inlineStr">
+        <is>
+          <t>Um bloco de gelo absorve o primeiro golpe físico.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -8209,7 +8630,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Casco</t>
+          <t>Defesa leve</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -8249,6 +8670,11 @@
           <t>Halves damage from Special moves.</t>
         </is>
       </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>Reduz pela metade o dano especial.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -8328,7 +8754,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -8368,6 +8794,11 @@
           <t>Prevents poison.</t>
         </is>
       </c>
+      <c r="O111" t="inlineStr">
+        <is>
+          <t>Impede envenenamento.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -8417,7 +8848,7 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -8457,6 +8888,11 @@
           <t>Bypasses Light Screen, Reflect, and Safeguard.</t>
         </is>
       </c>
+      <c r="O113" t="inlineStr">
+        <is>
+          <t>Atravessa barreiras como Reflect e Light Screen.</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -8516,6 +8952,11 @@
           <t>When this Pokémon faints from an opponent's move, that opponent takes damage equal to the HP this Pokémon had remaining.</t>
         </is>
       </c>
+      <c r="O114" t="inlineStr">
+        <is>
+          <t>Ao cair, causa dano igual ao HP que tinha.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -8535,7 +8976,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -8575,6 +9016,11 @@
           <t>Prevents flinching.</t>
         </is>
       </c>
+      <c r="O115" t="inlineStr">
+        <is>
+          <t>Impede recuar (flinch) e, nas gerações novas, também a Intimidação.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -8594,7 +9040,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -8634,6 +9080,11 @@
           <t>Prevents sleep.</t>
         </is>
       </c>
+      <c r="O116" t="inlineStr">
+        <is>
+          <t>Impede o sono.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -8698,6 +9149,11 @@
           <t>Lowers opponents' Attack one stage upon entering battle.</t>
         </is>
       </c>
+      <c r="O117" t="inlineStr">
+        <is>
+          <t>Reduz o Ataque dos rivais ao entrar em combate.</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -8717,7 +9173,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Poder bruto</t>
+          <t>Ataque reforçado</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -8757,6 +9213,11 @@
           <t>Boosts Attack in battle.</t>
         </is>
       </c>
+      <c r="O118" t="inlineStr">
+        <is>
+          <t>Aumenta o Ataque ao entrar em combate.</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -8816,6 +9277,11 @@
           <t>Damages attacking Pokémon for 1/8 their max HP on contact.</t>
         </is>
       </c>
+      <c r="O119" t="inlineStr">
+        <is>
+          <t>Machuca quem o atinge com contato.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -8880,6 +9346,11 @@
           <t>Strengthens punch-based moves to 1.2× their power.</t>
         </is>
       </c>
+      <c r="O120" t="inlineStr">
+        <is>
+          <t>Golpes de soco ficam mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -8939,6 +9410,11 @@
           <t>Raises Attack one stage upon taking damage from a Dark move.</t>
         </is>
       </c>
+      <c r="O121" t="inlineStr">
+        <is>
+          <t>Ataque sobe ao ser atingido por golpe Sombrio.</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -8958,7 +9434,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -8998,6 +9474,11 @@
           <t>Prevents accuracy from being lowered.</t>
         </is>
       </c>
+      <c r="O122" t="inlineStr">
+        <is>
+          <t>Impede que a precisão seja reduzida.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -9047,7 +9528,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -9087,6 +9568,11 @@
           <t>Protects against major status ailments during strong sunlight.</t>
         </is>
       </c>
+      <c r="O124" t="inlineStr">
+        <is>
+          <t>Protege de problemas de status sob sol forte.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -9151,6 +9637,11 @@
           <t>Evades Ground moves.</t>
         </is>
       </c>
+      <c r="O125" t="inlineStr">
+        <is>
+          <t>Flutua: imune a golpes de Terra.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -9275,6 +9766,11 @@
           <t>Redirects single-target Electric moves to this Pokémon where possible.  Absorbs Electric moves, raising Special Attack one stage.</t>
         </is>
       </c>
+      <c r="O128" t="inlineStr">
+        <is>
+          <t>Atrai golpes Elétricos e ganha Ataque Especial.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -9294,7 +9790,7 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
@@ -9334,6 +9830,11 @@
           <t>Prevents paralysis.</t>
         </is>
       </c>
+      <c r="O129" t="inlineStr">
+        <is>
+          <t>Impede paralisia.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -9398,6 +9899,11 @@
           <t>Contact changes the attacker's Ability to Lingering Aroma.</t>
         </is>
       </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>Troca a habilidade de quem faz contato.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -9457,6 +9963,11 @@
           <t>Damages opponents using leeching moves for as much as they would heal.</t>
         </is>
       </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>Quem rouba HP dele perde HP.</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -9521,6 +10032,11 @@
           <t>Sound-based moves become Water-type.</t>
         </is>
       </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>Golpes sonoros viram golpes de Água.</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -9540,7 +10056,7 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
@@ -9580,6 +10096,11 @@
           <t>This Pokémon's moves do not make contact.</t>
         </is>
       </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>Seus golpes nunca fazem contato.</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -9639,6 +10160,11 @@
           <t>Reflects most non-damaging moves back at their user.</t>
         </is>
       </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>Reflete golpes de status de volta.</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -9692,6 +10218,11 @@
           <t>Protects against damage not directly caused by a move.</t>
         </is>
       </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>Só sofre dano direto de golpes.</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -9741,7 +10272,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -9781,6 +10312,11 @@
           <t>Prevents freezing.</t>
         </is>
       </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>Impede congelamento.</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -9870,6 +10406,11 @@
           <t>Increases Defense to 1.5× with a major status ailment.</t>
         </is>
       </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>Defesa maior quando está com problema de status.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -9934,6 +10475,11 @@
           <t>Strengthens aura and pulse moves to 1.5× their power.</t>
         </is>
       </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>Golpes de pulso e aura ficam mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -9998,6 +10544,11 @@
           <t>The Pokémon can use its moves as if the weather were harsh sunlight.</t>
         </is>
       </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>Usa os golpes como se houvesse sol forte.</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -10017,7 +10568,7 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -10057,6 +10608,11 @@
           <t>This Pokémon's moves critical hit against poisoned targets.</t>
         </is>
       </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>Golpes sempre críticos contra alvos envenenados.</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -10106,7 +10662,7 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -10146,6 +10702,11 @@
           <t>The Pokémon ignores changes to opponents' evasiveness, its accuracy can't be lowered, and it can hit Ghost types with Normal- and Fighting-type moves.</t>
         </is>
       </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>Ignora a esquiva do alvo e não perde precisão.</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -10205,6 +10766,11 @@
           <t>Increases Special Attack to 1.5× when a friendly Pokémon has Plus or Minus.</t>
         </is>
       </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>Aumenta o Ataque Especial junto de um aliado Plus/Minus.</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -10264,6 +10830,11 @@
           <t>Reflects any stat-lowering effects.</t>
         </is>
       </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>Reflete efeitos que reduzem atributos.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -10328,6 +10899,11 @@
           <t>When this Pokémon enters battle, it changes the terrain to Misty Terrain.</t>
         </is>
       </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>Cria terreno de névoa ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -10347,7 +10923,7 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
@@ -10387,6 +10963,11 @@
           <t>Bypasses targets' abilities if they could hinder or prevent a move.</t>
         </is>
       </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>Ignora habilidades do alvo que atrapalhariam o golpe.</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -10446,6 +11027,11 @@
           <t>Raises a random stat two stages and lowers another one stage after each turn.</t>
         </is>
       </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>Todo turno sobe um atributo e reduz outro.</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -10510,6 +11096,11 @@
           <t>Absorbs Electric moves, raising Speed one stage.</t>
         </is>
       </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>Absorve golpes Elétricos e ganha Velocidade.</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -10569,6 +11160,11 @@
           <t>Raises Attack one stage upon KOing a Pokémon.</t>
         </is>
       </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>Ataque sobe ao derrotar um Pokémon.</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -10628,6 +11224,11 @@
           <t>Halves damage taken from full HP.</t>
         </is>
       </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>Com HP cheio, reduz pela metade o dano recebido.</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -10722,6 +11323,11 @@
           <t>Changes attacking Pokémon's abilities to Mummy on contact.</t>
         </is>
       </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>Troca a habilidade de quem faz contato por Mummy.</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -10811,6 +11417,11 @@
           <t>Cures any major status ailment upon switching out.</t>
         </is>
       </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>Cura problemas de status ao sair de campo.</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -10870,6 +11481,11 @@
           <t>Increases super-effective damage dealt to 1.25×.</t>
         </is>
       </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>Golpes super efetivos causam mais dano.</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -10919,7 +11535,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
@@ -10959,6 +11575,11 @@
           <t>Ensures all moves used by and against the Pokémon hit.</t>
         </is>
       </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>Todos os golpes (dele e contra ele) acertam.</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -11008,7 +11629,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
@@ -11048,6 +11669,11 @@
           <t>Prevents infatuation and protects against Captivate.</t>
         </is>
       </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>Impede paixão e provocação.</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -11142,6 +11768,11 @@
           <t>Turns the sunlight harsh when entering battle, and boosts Attack while active.</t>
         </is>
       </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>Invoca sol forte e aumenta o Ataque.</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -11161,7 +11792,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Casco</t>
+          <t>Defesa leve</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
@@ -11201,6 +11832,11 @@
           <t>Protects against damage from weather.</t>
         </is>
       </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>Protege de dano de clima e de golpes de pó.</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -11265,6 +11901,11 @@
           <t>Strengthens Grass moves to inflict 1.5× damage at 1/3 max HP or less.</t>
         </is>
       </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>Golpes de Planta ficam mais fortes com HP baixo.</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -11284,7 +11925,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
@@ -11324,6 +11965,11 @@
           <t>Prevents confusion.</t>
         </is>
       </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>Impede confusão.</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -11383,6 +12029,11 @@
           <t>Lets the bearer hit twice with damaging moves.  The second hit has half power.</t>
         </is>
       </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>Golpes batem duas vezes (a segunda com metade da força).</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -11442,6 +12093,11 @@
           <t>When hit by a move that makes direct contact, the Pokémon and the attacker will faint after three turns unless they switch out of battle.</t>
         </is>
       </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>Quem o atinge com contato cai em três turnos.</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -11521,7 +12177,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
@@ -11561,6 +12217,11 @@
           <t>When the Pokémon uses contact moves, it can hit even targets that are protecting themselves.</t>
         </is>
       </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>Golpes de contato atravessam a proteção do alvo.</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -11625,6 +12286,11 @@
           <t>Turns the bearer's Normal moves into Fairy moves and strengthens them to 1.3× their power.</t>
         </is>
       </c>
+      <c r="O172" t="inlineStr">
+        <is>
+          <t>Golpes Normais viram Fada, mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -11684,6 +12350,11 @@
           <t>Increases Special Attack to 1.5× when a friendly Pokémon has Plus or Minus.</t>
         </is>
       </c>
+      <c r="O173" t="inlineStr">
+        <is>
+          <t>Aumenta o Ataque Especial junto de um aliado Plus/Minus.</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -11743,6 +12414,11 @@
           <t>Heals for 1/8 max HP after each turn when poisoned in place of damage.</t>
         </is>
       </c>
+      <c r="O174" t="inlineStr">
+        <is>
+          <t>Recupera HP todo turno quando envenenado.</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -11807,6 +12483,11 @@
           <t>Has a 30% chance of poisoning attacking Pokémon on contact.</t>
         </is>
       </c>
+      <c r="O175" t="inlineStr">
+        <is>
+          <t>30% de chance de envenenar quem faz contato.</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -11871,6 +12552,11 @@
           <t>Pokémon poisoned by Pecharunt's moves will also become confused.</t>
         </is>
       </c>
+      <c r="O176" t="inlineStr">
+        <is>
+          <t>Alvos envenenados também ficam confusos.</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -11935,6 +12621,11 @@
           <t>Has a 30% chance of poisoning target Pokémon upon contact.</t>
         </is>
       </c>
+      <c r="O177" t="inlineStr">
+        <is>
+          <t>30% de chance de envenenar ao atacar com contato.</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -12024,6 +12715,11 @@
           <t>Just being next to the Pokémon powers up moves.</t>
         </is>
       </c>
+      <c r="O179" t="inlineStr">
+        <is>
+          <t>Aumenta o poder dos golpes de quem está ao lado.</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -12083,6 +12779,11 @@
           <t>Raises non-damaging moves' priority by one stage.</t>
         </is>
       </c>
+      <c r="O180" t="inlineStr">
+        <is>
+          <t>Golpes de status agem primeiro.</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -12147,6 +12848,11 @@
           <t>Increases the PP cost of moves targetting the Pokémon by one.</t>
         </is>
       </c>
+      <c r="O181" t="inlineStr">
+        <is>
+          <t>Faz os golpes contra ele gastarem mais PP.</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -12211,6 +12917,11 @@
           <t>Creates heavy rain, which has all the properties of Rain Dance, cannot be replaced, and causes damaging Fire moves to fail.</t>
         </is>
       </c>
+      <c r="O182" t="inlineStr">
+        <is>
+          <t>Invoca chuva forte ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -12270,6 +12981,11 @@
           <t>Reduces super-effective damage to 0.75×.</t>
         </is>
       </c>
+      <c r="O183" t="inlineStr">
+        <is>
+          <t>Reduz o dano de golpes super efetivos.</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -12349,7 +13065,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Poder bruto</t>
+          <t>Ataque reforçado</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
@@ -12389,6 +13105,11 @@
           <t>Raises highest stat in harsh sunlight, or if holding Booster Energy.</t>
         </is>
       </c>
+      <c r="O186" t="inlineStr">
+        <is>
+          <t>Aumenta o maior atributo sob sol forte.</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -12453,6 +13174,11 @@
           <t>When this Pokémon enters battle, it changes the terrain to Psychic Terrain.</t>
         </is>
       </c>
+      <c r="O187" t="inlineStr">
+        <is>
+          <t>Cria terreno psíquico ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -12517,6 +13243,11 @@
           <t>Boosts sound-based moves and halves damage from the same moves.</t>
         </is>
       </c>
+      <c r="O188" t="inlineStr">
+        <is>
+          <t>Golpes sonoros ficam mais fortes e causam menos dano a ele.</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -12536,7 +13267,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Poder bruto</t>
+          <t>Ataque reforçado</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
@@ -12576,6 +13307,11 @@
           <t>Doubles Attack in battle.</t>
         </is>
       </c>
+      <c r="O189" t="inlineStr">
+        <is>
+          <t>Dobra o Ataque.</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -12595,7 +13331,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
@@ -12635,6 +13371,11 @@
           <t>Protects from status conditions and halves damage from Ghost-type moves.</t>
         </is>
       </c>
+      <c r="O190" t="inlineStr">
+        <is>
+          <t>Protege de problemas de status e reduz dano Fantasma.</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -12654,7 +13395,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Poder bruto</t>
+          <t>Ataque reforçado</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
@@ -12694,6 +13435,11 @@
           <t>Raises highest stat on Electric Terrain, or if holding Booster Energy.</t>
         </is>
       </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>Aumenta o maior atributo em terreno elétrico.</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -12758,6 +13504,11 @@
           <t>Opposing Pokémon cannot use priority attacks.</t>
         </is>
       </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>Impede os rivais de usar golpes com prioridade.</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -12817,6 +13568,11 @@
           <t>Increases Speed to 1.5× with a major status ailment.</t>
         </is>
       </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>Velocidade maior quando está com problema de status.</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -12876,6 +13632,11 @@
           <t>Heals for 1/16 max HP after each turn during rain.</t>
         </is>
       </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>Recupera um pouco de HP todo turno na chuva.</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -12935,6 +13696,11 @@
           <t>Raises Speed one stage upon being hit by a Dark, Ghost, or Bug move.</t>
         </is>
       </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>Ganha Velocidade ao ser atingido por golpes Sombrios, Fantasmas ou de Inseto.</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -12994,6 +13760,11 @@
           <t>When an ally faints, this Pokémon gains its Ability.</t>
         </is>
       </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>Ao cair um aliado, ganha a habilidade dele.</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -13058,6 +13829,11 @@
           <t>Strengthens recoil moves to 1.2× their power.</t>
         </is>
       </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>Golpes com recuo ficam mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -13122,6 +13898,11 @@
           <t>Turns the bearer's Normal moves into Ice moves and strengthens them to 1.3× their power.</t>
         </is>
       </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>Golpes Normais viram Gelo, mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -13181,6 +13962,11 @@
           <t>Heals for 1/3 max HP upon switching out.</t>
         </is>
       </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>Recupera 1/3 do HP ao sair de campo.</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -13290,7 +14076,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>Casco</t>
+          <t>Defesa leve</t>
         </is>
       </c>
       <c r="E203" t="inlineStr">
@@ -13330,6 +14116,11 @@
           <t>Protects against recoil damage.</t>
         </is>
       </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>Impede o dano de recuo dos próprios golpes.</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -13394,6 +14185,11 @@
           <t>Powers up Rock-type moves.</t>
         </is>
       </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>Golpes de Pedra ficam mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -13453,6 +14249,11 @@
           <t>Damages attacking Pokémon for 1/8 their max HP on contact.</t>
         </is>
       </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>Machuca quem o atinge com contato.</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -13547,6 +14348,11 @@
           <t>Strengthens Rock, Ground, and Steel moves to 1.3× their power during a sandstorm.  Protects against sandstorm damage.</t>
         </is>
       </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>Golpes de Pedra, Terra e Aço ficam mais fortes na tempestade de areia.</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -13606,6 +14412,11 @@
           <t>Doubles Speed during a sandstorm.  Protects against sandstorm damage.</t>
         </is>
       </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>Dobra a Velocidade na tempestade de areia.</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -13700,6 +14511,11 @@
           <t>Summons a sandstorm that lasts indefinitely upon entering battle.</t>
         </is>
       </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>Invoca tempestade de areia ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -13759,6 +14575,11 @@
           <t>Increases evasion to 1.25× during a sandstorm.  Protects against sandstorm damage.</t>
         </is>
       </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>Aumenta a esquiva na tempestade de areia.</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -13823,6 +14644,11 @@
           <t>Absorbs Grass moves, raising Attack one stage.</t>
         </is>
       </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>Absorve golpes de Planta e ganha Ataque.</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -13872,7 +14698,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E214" t="inlineStr">
@@ -13912,6 +14738,11 @@
           <t>Lets the Pokémon's Normal and Fighting moves hit Ghost Pokémon.</t>
         </is>
       </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>Golpes Normais e Lutadores acertam Fantasmas.</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -14006,6 +14837,11 @@
           <t>Turns the ground into Grassy Terrain when the Pokémon is hit by an attack.</t>
         </is>
       </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>Cria terreno de grama ao ser atingido.</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -14095,6 +14931,11 @@
           <t>When this Pokémon has full HP, regular damage from moves is halved.</t>
         </is>
       </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>Com HP cheio, reduz pela metade o dano recebido.</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -14189,6 +15030,11 @@
           <t>Powers up slicing moves.</t>
         </is>
       </c>
+      <c r="O220" t="inlineStr">
+        <is>
+          <t>Golpes cortantes ficam mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -14248,6 +15094,11 @@
           <t>Has a 33% chance of curing any major status ailment after each turn.</t>
         </is>
       </c>
+      <c r="O221" t="inlineStr">
+        <is>
+          <t>Chance de curar status todo turno.</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -14312,6 +15163,11 @@
           <t>Strengthens moves with extra effects to 1.3× their power, but prevents their extra effects.</t>
         </is>
       </c>
+      <c r="O222" t="inlineStr">
+        <is>
+          <t>Golpes com efeito extra ficam mais fortes, mas perdem o efeito.</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -14331,7 +15187,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>Casco</t>
+          <t>Defesa leve</t>
         </is>
       </c>
       <c r="E223" t="inlineStr">
@@ -14371,6 +15227,11 @@
           <t>Protects against critical hits.</t>
         </is>
       </c>
+      <c r="O223" t="inlineStr">
+        <is>
+          <t>Impede golpes críticos.</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -14390,7 +15251,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E224" t="inlineStr">
@@ -14430,6 +15291,11 @@
           <t>Protects against incoming moves' extra effects.</t>
         </is>
       </c>
+      <c r="O224" t="inlineStr">
+        <is>
+          <t>Bloqueia os efeitos extras de golpes recebidos.</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -14549,6 +15415,11 @@
           <t>Extends two-to-five-hit moves and Triple Kick to their full length every time.</t>
         </is>
       </c>
+      <c r="O227" t="inlineStr">
+        <is>
+          <t>Golpes de vários acertos sempre acertam o máximo.</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -14638,6 +15509,11 @@
           <t>During Hail, this Pokémon has double Speed.</t>
         </is>
       </c>
+      <c r="O229" t="inlineStr">
+        <is>
+          <t>Dobra a Velocidade no granizo.</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -14657,7 +15533,7 @@
       </c>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
@@ -14697,6 +15573,11 @@
           <t>Strengthens critical hits to inflict 3× damage rather than 2×.</t>
         </is>
       </c>
+      <c r="O230" t="inlineStr">
+        <is>
+          <t>Golpes críticos causam ainda mais dano.</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -14756,6 +15637,11 @@
           <t>Increases evasion to 1.25× during hail.  Protects against hail damage.</t>
         </is>
       </c>
+      <c r="O231" t="inlineStr">
+        <is>
+          <t>Aumenta a esquiva no granizo.</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -14820,6 +15706,11 @@
           <t>Summons hail that lasts indefinitely upon entering battle.</t>
         </is>
       </c>
+      <c r="O232" t="inlineStr">
+        <is>
+          <t>Invoca granizo ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -14839,7 +15730,7 @@
       </c>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Poder bruto</t>
+          <t>Ataque reforçado</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
@@ -14879,6 +15770,11 @@
           <t>Increases Special Attack to 1.5× but costs 1/8 max HP after each turn during strong sunlight.</t>
         </is>
       </c>
+      <c r="O233" t="inlineStr">
+        <is>
+          <t>Ataque Especial maior sob sol forte, com custo de HP.</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -14938,6 +15834,11 @@
           <t>Decreases damage taken from super-effective moves by 1/4.</t>
         </is>
       </c>
+      <c r="O234" t="inlineStr">
+        <is>
+          <t>Reduz o dano de golpes super efetivos.</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -14997,6 +15898,11 @@
           <t>This Pokémon's Special Attack rises by one stage every time any Pokémon faints.</t>
         </is>
       </c>
+      <c r="O235" t="inlineStr">
+        <is>
+          <t>Ataque Especial sobe sempre que qualquer Pokémon cai.</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -15016,7 +15922,7 @@
       </c>
       <c r="D236" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
@@ -15056,6 +15962,11 @@
           <t>Protects against sound-based moves.</t>
         </is>
       </c>
+      <c r="O236" t="inlineStr">
+        <is>
+          <t>Bloqueia golpes sonoros.</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -15115,6 +16026,11 @@
           <t>Raises Speed one stage after each turn.</t>
         </is>
       </c>
+      <c r="O237" t="inlineStr">
+        <is>
+          <t>A Velocidade sobe um pouco a cada turno.</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -15174,6 +16090,11 @@
           <t>When the Pokémon takes damage from a move, it burns the attacker.</t>
         </is>
       </c>
+      <c r="O238" t="inlineStr">
+        <is>
+          <t>Queima quem o atinge.</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -15193,7 +16114,7 @@
       </c>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
@@ -15233,6 +16154,11 @@
           <t>This Pokémon's moves have double power against Pokémon that switched in this turn.</t>
         </is>
       </c>
+      <c r="O239" t="inlineStr">
+        <is>
+          <t>Dobra o dano contra quem acabou de entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -15352,6 +16278,11 @@
           <t>Raises this Pokémon's Defense by one stage when it takes damage from a move.</t>
         </is>
       </c>
+      <c r="O242" t="inlineStr">
+        <is>
+          <t>Defesa sobe ao ser atingido.</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -15446,6 +16377,11 @@
           <t>Has a 30% chance of paralyzing attacking Pokémon on contact.</t>
         </is>
       </c>
+      <c r="O244" t="inlineStr">
+        <is>
+          <t>30% de chance de paralisar quem faz contato.</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
@@ -15535,6 +16471,11 @@
           <t>Boosts the Speed stat drastically when the Pokémon is hit by a Fire- or Water-type move.</t>
         </is>
       </c>
+      <c r="O246" t="inlineStr">
+        <is>
+          <t>Velocidade sobe muito ao ser atingido por Fogo ou Água.</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
@@ -15599,6 +16540,11 @@
           <t>This Pokémon's Steel moves have 1.5× power.</t>
         </is>
       </c>
+      <c r="O247" t="inlineStr">
+        <is>
+          <t>Golpes de Aço ficam mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
@@ -15663,6 +16609,11 @@
           <t>Powers up ally Pokémon's Steel-type moves.</t>
         </is>
       </c>
+      <c r="O248" t="inlineStr">
+        <is>
+          <t>Golpes de Aço dos aliados ficam mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -15727,6 +16678,11 @@
           <t>Has a 10% chance of making target Pokémon flinch with each hit.</t>
         </is>
       </c>
+      <c r="O249" t="inlineStr">
+        <is>
+          <t>10% de chance de fazer o alvo recuar.</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
@@ -15821,6 +16777,11 @@
           <t>Redirects single-target Water moves to this Pokémon where possible.  Absorbs Water moves, raising Special Attack one stage.</t>
         </is>
       </c>
+      <c r="O251" t="inlineStr">
+        <is>
+          <t>Atrai golpes de Água e ganha Ataque Especial.</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
@@ -15885,6 +16846,11 @@
           <t>Strengthens biting moves to 1.5× their power.</t>
         </is>
       </c>
+      <c r="O252" t="inlineStr">
+        <is>
+          <t>Golpes de mordida ficam mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
@@ -15938,6 +16904,11 @@
           <t>Prevents being KOed from full HP, leaving 1 HP instead.  Protects against the one-hit KO moves regardless of HP.</t>
         </is>
       </c>
+      <c r="O253" t="inlineStr">
+        <is>
+          <t>Não é derrotado de uma vez com HP cheio.</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
@@ -15987,7 +16958,7 @@
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
@@ -16027,6 +16998,11 @@
           <t>Raises moves' critical hit rates one stage.</t>
         </is>
       </c>
+      <c r="O255" t="inlineStr">
+        <is>
+          <t>Aumenta a chance de golpe crítico.</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
@@ -16091,6 +17067,11 @@
           <t xml:space="preserve">Once per battle, when a Pokémon with Supersweet Syrup enters the battle, it lowers the evasion stat of all adjacent opponents by one stage. </t>
         </is>
       </c>
+      <c r="O256" t="inlineStr">
+        <is>
+          <t>Reduz a esquiva dos rivais ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
@@ -16150,6 +17131,11 @@
           <t>Attack and Special Attack are boosted for each party Pokémon that has been defeated.</t>
         </is>
       </c>
+      <c r="O257" t="inlineStr">
+        <is>
+          <t>Ataque e Ataque Especial sobem por aliado derrotado.</t>
+        </is>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
@@ -16214,6 +17200,11 @@
           <t>Strengthens Bug moves to inflict 1.5× damage at 1/3 max HP or less.</t>
         </is>
       </c>
+      <c r="O258" t="inlineStr">
+        <is>
+          <t>Golpes de Inseto ficam mais fortes com HP baixo.</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -16273,6 +17264,11 @@
           <t>Prevents friendly Pokémon from sleeping.</t>
         </is>
       </c>
+      <c r="O259" t="inlineStr">
+        <is>
+          <t>Impede os aliados de dormir.</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -16332,6 +17328,11 @@
           <t>Doubles Speed during rain.</t>
         </is>
       </c>
+      <c r="O260" t="inlineStr">
+        <is>
+          <t>Dobra a Velocidade na chuva.</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
@@ -16396,6 +17397,11 @@
           <t>Lowers Defense of all Pokémon except itself.</t>
         </is>
       </c>
+      <c r="O261" t="inlineStr">
+        <is>
+          <t>Reduz a Defesa de todos os outros Pokémon.</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -16455,6 +17461,11 @@
           <t>Passes the bearer's held item to an ally when the ally uses up its item.</t>
         </is>
       </c>
+      <c r="O262" t="inlineStr">
+        <is>
+          <t>Passa o item para um aliado que ficou sem.</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -16514,6 +17525,11 @@
           <t>Copies burns, paralysis, and poison received onto the Pokémon that inflicted them.</t>
         </is>
       </c>
+      <c r="O263" t="inlineStr">
+        <is>
+          <t>Devolve queimadura, paralisia e veneno a quem os causou.</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -16578,6 +17594,11 @@
           <t>Lowers Attack of all Pokémon except itself.</t>
         </is>
       </c>
+      <c r="O264" t="inlineStr">
+        <is>
+          <t>Reduz o Ataque de todos os outros Pokémon.</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -16637,6 +17658,11 @@
           <t>Doubles evasion when confused.</t>
         </is>
       </c>
+      <c r="O265" t="inlineStr">
+        <is>
+          <t>Dobra a esquiva quando confuso.</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -16701,6 +17727,11 @@
           <t>Strengthens moves of 60 base power or less to 1.5× their power.</t>
         </is>
       </c>
+      <c r="O266" t="inlineStr">
+        <is>
+          <t>Golpes fracos (até 60 de poder) ficam 50% mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
@@ -16790,6 +17821,11 @@
           <t>All damage-dealing moves that hit the Pokémon when its HP is full will not be very effective.</t>
         </is>
       </c>
+      <c r="O268" t="inlineStr">
+        <is>
+          <t>Com HP cheio, nenhum golpe é super efetivo contra ele.</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -16869,7 +17905,7 @@
       </c>
       <c r="D271" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E271" t="inlineStr">
@@ -16909,6 +17945,11 @@
           <t>Bypasses targets' abilities if they could hinder or prevent moves.</t>
         </is>
       </c>
+      <c r="O271" t="inlineStr">
+        <is>
+          <t>Ignora habilidades do alvo que atrapalhariam o golpe.</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -16968,6 +18009,11 @@
           <t>Raises Attack when hit by a Fire-type move. Cannot be burned.</t>
         </is>
       </c>
+      <c r="O272" t="inlineStr">
+        <is>
+          <t>Ataque sobe ao ser atingido por Fogo e não queima.</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
@@ -17032,6 +18078,11 @@
           <t>Halves damage from Fire and Ice moves.</t>
         </is>
       </c>
+      <c r="O273" t="inlineStr">
+        <is>
+          <t>Reduz pela metade o dano de Fogo e Gelo.</t>
+        </is>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
@@ -17091,6 +18142,11 @@
           <t>Doubles damage inflicted with not-very-effective moves.</t>
         </is>
       </c>
+      <c r="O274" t="inlineStr">
+        <is>
+          <t>Golpes pouco efetivos causam o dobro de dano.</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -17155,6 +18211,11 @@
           <t>Strengthens Water moves to inflict 1.5× damage at 1/3 max HP or less.</t>
         </is>
       </c>
+      <c r="O275" t="inlineStr">
+        <is>
+          <t>Golpes de Água ficam mais fortes com HP baixo.</t>
+        </is>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
@@ -17219,6 +18280,11 @@
           <t>Strengthens moves that make contact to 1.33× their power.</t>
         </is>
       </c>
+      <c r="O276" t="inlineStr">
+        <is>
+          <t>Golpes de contato ficam mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
@@ -17278,6 +18344,11 @@
           <t>Increases Attack to 1.5× when poisoned.</t>
         </is>
       </c>
+      <c r="O277" t="inlineStr">
+        <is>
+          <t>Ataque maior quando envenenado.</t>
+        </is>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
@@ -17342,6 +18413,11 @@
           <t>May cause bad poisoning when the Pokémon hits an opponent with a move.</t>
         </is>
       </c>
+      <c r="O278" t="inlineStr">
+        <is>
+          <t>Pode envenenar gravemente ao atingir um rival.</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -17401,6 +18477,11 @@
           <t>Scatters poison spikes at the feet of the opposing team when the Pokémon takes damage from physical moves.</t>
         </is>
       </c>
+      <c r="O279" t="inlineStr">
+        <is>
+          <t>Espalha espinhos venenosos ao ser atingido.</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -17495,6 +18576,11 @@
           <t>Powers up Electric-type moves.</t>
         </is>
       </c>
+      <c r="O281" t="inlineStr">
+        <is>
+          <t>Golpes Elétricos ficam mais fortes.</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
@@ -17554,6 +18640,11 @@
           <t>This Pokémon's healing moves have their priority increased by 3.</t>
         </is>
       </c>
+      <c r="O282" t="inlineStr">
+        <is>
+          <t>Golpes de cura agem primeiro.</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -17603,7 +18694,7 @@
       </c>
       <c r="D284" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E284" t="inlineStr">
@@ -17643,6 +18734,11 @@
           <t>Bypasses targets' abilities if they could hinder or prevent moves.</t>
         </is>
       </c>
+      <c r="O284" t="inlineStr">
+        <is>
+          <t>Ignora habilidades do alvo que atrapalhariam o golpe.</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
@@ -17702,6 +18798,11 @@
           <t>Ignores other Pokémon's stat modifiers for damage and accuracy calculation.</t>
         </is>
       </c>
+      <c r="O285" t="inlineStr">
+        <is>
+          <t>Ignora as mudanças de atributo do rival.</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
@@ -17761,6 +18862,11 @@
           <t>Doubles Speed upon using or losing a held item.</t>
         </is>
       </c>
+      <c r="O286" t="inlineStr">
+        <is>
+          <t>Dobra a Velocidade ao usar ou perder o item.</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
@@ -17825,6 +18931,11 @@
           <t>Prevents opposing Pokémon from eating held Berries.</t>
         </is>
       </c>
+      <c r="O287" t="inlineStr">
+        <is>
+          <t>Impede os rivais de comer frutas.</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
@@ -17844,7 +18955,7 @@
       </c>
       <c r="D288" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E288" t="inlineStr">
@@ -17884,6 +18995,11 @@
           <t>Contact moves can strike through Protect/Detect.</t>
         </is>
       </c>
+      <c r="O288" t="inlineStr">
+        <is>
+          <t>Golpes de contato atravessam a proteção do alvo.</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -17948,6 +19064,11 @@
           <t>Lowers Special Attack of all Pokémon except itself.</t>
         </is>
       </c>
+      <c r="O289" t="inlineStr">
+        <is>
+          <t>Reduz o Ataque Especial de todos os outros Pokémon.</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
@@ -17967,7 +19088,7 @@
       </c>
       <c r="D290" t="inlineStr">
         <is>
-          <t>Quebra-defesas</t>
+          <t>Golpe certeiro</t>
         </is>
       </c>
       <c r="E290" t="inlineStr">
@@ -18007,6 +19128,11 @@
           <t>Increases moves' accuracy to 1.1× for friendly Pokémon.</t>
         </is>
       </c>
+      <c r="O290" t="inlineStr">
+        <is>
+          <t>Aumenta a precisão da equipe.</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
@@ -18026,7 +19152,7 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
@@ -18066,6 +19192,11 @@
           <t>Prevents sleep.</t>
         </is>
       </c>
+      <c r="O291" t="inlineStr">
+        <is>
+          <t>Impede o sono.</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
@@ -18130,6 +19261,11 @@
           <t>Absorbs Electric moves, healing for 1/4 max HP.</t>
         </is>
       </c>
+      <c r="O292" t="inlineStr">
+        <is>
+          <t>Recupera HP ao ser atingido por golpes Elétricos.</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
@@ -18194,6 +19330,11 @@
           <t>Swaps abilities with opponents on contact.</t>
         </is>
       </c>
+      <c r="O293" t="inlineStr">
+        <is>
+          <t>Troca de habilidade com quem faz contato.</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -18258,6 +19399,11 @@
           <t>Absorbs Water moves, healing for 1/4 max HP.</t>
         </is>
       </c>
+      <c r="O294" t="inlineStr">
+        <is>
+          <t>Recupera HP ao ser atingido por golpes de Água.</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -18322,6 +19468,11 @@
           <t>Halves damage from Fire moves, doubles damage of Water moves, and prevents burns.</t>
         </is>
       </c>
+      <c r="O295" t="inlineStr">
+        <is>
+          <t>Reduz o dano de Fogo, dobra o de Água e impede queimaduras.</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -18381,6 +19532,11 @@
           <t>Raises this Pokémon's Defense by two stages when it's hit by a Water move.</t>
         </is>
       </c>
+      <c r="O296" t="inlineStr">
+        <is>
+          <t>Defesa sobe muito ao ser atingido por Água.</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -18400,7 +19556,7 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
@@ -18440,6 +19596,11 @@
           <t>Prevents burns.</t>
         </is>
       </c>
+      <c r="O297" t="inlineStr">
+        <is>
+          <t>Impede queimaduras.</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -18499,6 +19660,11 @@
           <t>Raises Speed and lowers Defense by one stage each upon being hit by a physical move.</t>
         </is>
       </c>
+      <c r="O298" t="inlineStr">
+        <is>
+          <t>Ao ser atingido por golpe físico, perde Defesa e ganha Velocidade.</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -18563,6 +19729,11 @@
           <t>Immune to Fire-type moves, and Defense is sharply boosted.</t>
         </is>
       </c>
+      <c r="O299" t="inlineStr">
+        <is>
+          <t>Imune a Fogo e ganha muita Defesa.</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
@@ -18582,7 +19753,7 @@
       </c>
       <c r="D300" t="inlineStr">
         <is>
-          <t>Corpo limpo</t>
+          <t>Resistência a debuff</t>
         </is>
       </c>
       <c r="E300" t="inlineStr">
@@ -18622,6 +19793,11 @@
           <t>Prevents stats from being lowered by other Pokémon.</t>
         </is>
       </c>
+      <c r="O300" t="inlineStr">
+        <is>
+          <t>Impede que outros Pokémon reduzam seus atributos.</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -18681,6 +19857,11 @@
           <t>This Pokémon automatically switches out when its HP drops below half.</t>
         </is>
       </c>
+      <c r="O301" t="inlineStr">
+        <is>
+          <t>Sai de campo quando o HP cai abaixo da metade.</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
@@ -18740,6 +19921,11 @@
           <t>When hit by a wind move, the power of the next Electric-type move it uses is doubled.</t>
         </is>
       </c>
+      <c r="O302" t="inlineStr">
+        <is>
+          <t>Ao ser atingido por vento, o próximo golpe Elétrico dobra de poder.</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
@@ -18804,6 +19990,11 @@
           <t>Gives immunity to wind moves, and causes the Pokémon's Attack to increase by one stage when hit by one.</t>
         </is>
       </c>
+      <c r="O303" t="inlineStr">
+        <is>
+          <t>Imune a golpes de vento e ganha Ataque.</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -18863,6 +20054,11 @@
           <t>Protects against damaging moves that are not super effective.</t>
         </is>
       </c>
+      <c r="O304" t="inlineStr">
+        <is>
+          <t>Só golpes super efetivos o machucam.</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
@@ -18920,6 +20116,11 @@
       <c r="N305" t="inlineStr">
         <is>
           <t>Lowers incoming non-damaging moves' base accuracy to exactly 50%.</t>
+        </is>
+      </c>
+      <c r="O305" t="inlineStr">
+        <is>
+          <t>Golpes de status contra ele erram mais.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: todas as habilidades passam a ter efeito positivo (5 efeitos novos: anula bonus rivais, pesadelo, aquecimento, golpe feliz, roubo de vida); quem pode usar da pedra respeita o painel
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/habilidades-passivas-mascotes.xlsx
+++ b/docs/habilidades-passivas-mascotes.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2360,6 +2360,205 @@
         <is>
           <t>-</t>
         </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>ANULAR_BONUS</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Anula bônus rivais</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Nas 3 primeiras rodadas, anula os bônus de Ambiente e de Aura dos rivais.</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>3</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>PESADELO</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Pesadelo</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Controle</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Nas 3 primeiras rodadas, cada rival perde {rng} do HP máximo no início da rodada.</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>3</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>2</v>
+      </c>
+      <c r="I49" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>AQUECIMENTO</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Aquecimento</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Nas 2 primeiras rodadas recebe {rng} menos dano; depois, seus 3 golpes seguintes causam {rng} mais dano.</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>3</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>6</v>
+      </c>
+      <c r="I50" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>GOLPE_FELIZ</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Golpe feliz</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>30% de chance de o golpe causar {rng} mais dano.</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>3</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>8</v>
+      </c>
+      <c r="I51" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>VAMPIRISMO</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Roubo de vida</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Recupera {rng} do dano causado.</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>3</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>6</v>
+      </c>
+      <c r="I52" t="n">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -2680,12 +2879,36 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Anula bônus rivais</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ANULAR_BONUS</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
+          <t>Nas 3 primeiras rodadas, anula os bônus de Ambiente e de Aura dos rivais.</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Instinto</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -2696,6 +2919,11 @@
           <t>Negates all effects of weather, but does not prevent the weather itself.</t>
         </is>
       </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Anula os efeitos de clima.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2902,13 +3130,43 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Armadura de tipos</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>ARMADURA</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Golpes com vantagem de tipo contra este mascote causam 6% a 20% menos dano.</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>6</v>
+      </c>
+      <c r="L9" t="n">
+        <v>20</v>
       </c>
       <c r="M9" t="n">
         <v>13</v>
@@ -2918,6 +3176,11 @@
           <t>Notifies all trainers upon entering battle if an opponent has a super-effective move, Self-Destruct, Explosion, or a one-hit KO move.</t>
         </is>
       </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Avisa se o rival tem um golpe super efetivo.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2932,13 +3195,47 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Controle</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Intimidação</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>INTIMIDACAO</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Agilidade</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Início da luta</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Reduz Agilidade de todos os rivais em 4% a 12%.</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Carisma</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>4</v>
+      </c>
+      <c r="L10" t="n">
+        <v>12</v>
       </c>
       <c r="M10" t="n">
         <v>3</v>
@@ -2948,6 +3245,11 @@
           <t>Prevents opponents from fleeing or switching out.  Eluded by Flying-types and Pokémon in the air.</t>
         </is>
       </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Impede os rivais de fugir ou trocar.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -3223,12 +3525,36 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Anula bônus rivais</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>ANULAR_BONUS</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
+          <t>Nas 3 primeiras rodadas, anula os bônus de Ambiente e de Aura dos rivais.</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Instinto</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -3239,6 +3565,11 @@
           <t>Makes Dark Aura and Fairy Aura weaken moves of their respective types.</t>
         </is>
       </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Inverte e enfraquece as auras Sombria e de Fada.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3317,13 +3648,43 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Controle</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Pesadelo</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PESADELO</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Nas 3 primeiras rodadas, cada rival perde 2% a 6% do HP máximo no início da rodada.</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>3</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L17" t="n">
+        <v>6</v>
       </c>
       <c r="M17" t="n">
         <v>1</v>
@@ -3333,6 +3694,11 @@
           <t>Damages sleeping opponents for 1/8 their max HP after each turn.</t>
         </is>
       </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Machuca rivais dormindo a cada turno.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -3347,13 +3713,43 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Cura gradual</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>CURA_GRADUAL</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Cura 3% a 10% do HP máximo.</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>3</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>3</v>
+      </c>
+      <c r="L18" t="n">
+        <v>10</v>
       </c>
       <c r="M18" t="n">
         <v>1</v>
@@ -3363,6 +3759,11 @@
           <t>If the Pokémon is not holding an item, it will fetch the Poké Ball from the first failed throw of the battle.</t>
         </is>
       </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Recupera a Poké Bola de uma captura que falhou.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4219,12 +4620,36 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Anula bônus rivais</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>ANULAR_BONUS</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
+          <t>Nas 3 primeiras rodadas, anula os bônus de Ambiente e de Aura dos rivais.</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>3</v>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Instinto</t>
         </is>
       </c>
       <c r="M32" t="n">
@@ -4235,6 +4660,11 @@
           <t>Negates all effects of weather, but does not prevent the weather itself.</t>
         </is>
       </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>Anula os efeitos de clima.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4249,13 +4679,43 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Defesa leve</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>CASCO</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Golpes causam 4% a 12% menos dano.</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>3</v>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>4</v>
+      </c>
+      <c r="L33" t="n">
+        <v>12</v>
       </c>
       <c r="M33" t="n">
         <v>1</v>
@@ -4265,6 +4725,11 @@
           <t>Changes type to match when hit by a damaging move.</t>
         </is>
       </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>Muda de tipo para o do golpe que o atingiu.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4279,13 +4744,43 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Resistência a debuff</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>CORPO_LIMPO</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Ao receber debuff</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Debuffs recebidos ficam 8% a 20% menores.</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>3</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>8</v>
+      </c>
+      <c r="L34" t="n">
+        <v>20</v>
       </c>
       <c r="M34" t="n">
         <v>1</v>
@@ -4295,6 +4790,11 @@
           <t>This Pokémon always  acts as though it were Asleep.</t>
         </is>
       </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>Age sempre como se estivesse dormindo (imune a status).</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4309,13 +4809,43 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Reforço</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>REFORCO</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Ao aplicar buff</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>O buff dado a aliados (Encorajador ou Batedor) fica 6% a 20% maior.</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
+        <v>2</v>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Carisma</t>
+        </is>
+      </c>
+      <c r="K35" t="n">
+        <v>6</v>
+      </c>
+      <c r="L35" t="n">
+        <v>20</v>
       </c>
       <c r="M35" t="n">
         <v>3</v>
@@ -4325,6 +4855,11 @@
           <t>Goes inside the mouth of an ally Dondozo if one is on the field.</t>
         </is>
       </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>Entra na boca de um Dondozo aliado.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4467,13 +5002,43 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Adversidade</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>ADVERSIDADE</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Ao receber debuff</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Ao ter um atributo reduzido, o próximo golpe causa 8% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>2</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K38" t="n">
+        <v>8</v>
+      </c>
+      <c r="L38" t="n">
+        <v>20</v>
       </c>
       <c r="M38" t="n">
         <v>13</v>
@@ -4483,6 +5048,11 @@
           <t>Inverts stat changes.</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Inverte as mudanças de atributo.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4901,12 +5471,36 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Sem efeito colateral</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>IMUNE_INDIRETO</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Passivo</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
+          <t>Não sofre dano de reflexo (Espinhos, Último suspiro) nem de efeitos indiretos de habilidades.</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="M45" t="n">
@@ -4917,6 +5511,11 @@
           <t>Prevents Self-Destruct, Explosion, and Aftermath from working while the Pokémon is in battle.</t>
         </is>
       </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>Impede explosões em campo.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4931,13 +5530,43 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Golpe duplo</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>GOLPE_DUPLO</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>O golpe ganha um segundo impacto de 6% a 20% do dano.</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>2</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K46" t="n">
+        <v>6</v>
+      </c>
+      <c r="L46" t="n">
+        <v>20</v>
       </c>
       <c r="M46" t="n">
         <v>4</v>
@@ -4947,6 +5576,11 @@
           <t>Whenever another Pokémon uses a dance move, this Pokémon will use the same move immediately afterwards.</t>
         </is>
       </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>Repete golpes de dança que vê.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5163,13 +5797,43 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Fúria</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>FURIA</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>HP baixo (abaixo de 33%)</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Os golpes causam 6% a 18% mais dano.</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>2</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K50" t="n">
+        <v>6</v>
+      </c>
+      <c r="L50" t="n">
+        <v>18</v>
       </c>
       <c r="M50" t="n">
         <v>2</v>
@@ -5179,6 +5843,11 @@
           <t>Halves Attack and Special Attack at 50% max HP or less.</t>
         </is>
       </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>Perde força quando o HP cai abaixo da metade.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5863,13 +6532,43 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Purificação</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>PURIFICACAO</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Ao remover debuff</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>No início da rodada, reduz em 6% a 20% o maior debuff do próprio mascote.</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>2</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>Carisma</t>
+        </is>
+      </c>
+      <c r="K61" t="n">
+        <v>6</v>
+      </c>
+      <c r="L61" t="n">
+        <v>20</v>
       </c>
       <c r="M61" t="n">
         <v>16</v>
@@ -5879,6 +6578,11 @@
           <t>Makes sleep pass twice as quickly.</t>
         </is>
       </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>Acorda do sono mais rápido.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -6893,13 +7597,43 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Vantagem ampliada</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>VANTAGEM</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Golpes com vantagem de tipo causam 6% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
+        <v>2</v>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K77" t="n">
+        <v>6</v>
+      </c>
+      <c r="L77" t="n">
+        <v>20</v>
       </c>
       <c r="M77" t="n">
         <v>3</v>
@@ -6909,6 +7643,11 @@
           <t>Changes Castform's type and form to match the weather.</t>
         </is>
       </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>Muda de tipo e forma conforme o clima.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6923,13 +7662,43 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Análise</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>ANALISE</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Início da luta</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>O primeiro golpe contra o rival de menor Vitalidade causa 6% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
+        <v>1</v>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K78" t="n">
+        <v>6</v>
+      </c>
+      <c r="L78" t="n">
+        <v>20</v>
       </c>
       <c r="M78" t="n">
         <v>6</v>
@@ -6939,6 +7708,11 @@
           <t>Reveals the opponents' strongest move upon entering battle.</t>
         </is>
       </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>Revela o golpe mais forte do rival ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -7017,13 +7791,43 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Análise</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>ANALISE</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Início da luta</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>O primeiro golpe contra o rival de menor Vitalidade causa 6% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>1</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K80" t="n">
+        <v>6</v>
+      </c>
+      <c r="L80" t="n">
+        <v>20</v>
       </c>
       <c r="M80" t="n">
         <v>36</v>
@@ -7033,6 +7837,11 @@
           <t>Reveals an opponent's held item upon entering battle.</t>
         </is>
       </c>
+      <c r="O80" t="inlineStr">
+        <is>
+          <t>Revela o item do rival ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -7239,13 +8048,43 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Regeneração</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>REGENERACAO</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>HP baixo (abaixo de 50%)</t>
         </is>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Recupera 8% a 20% do HP máximo.</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
+        <v>1</v>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K84" t="n">
+        <v>8</v>
+      </c>
+      <c r="L84" t="n">
+        <v>20</v>
       </c>
       <c r="M84" t="n">
         <v>32</v>
@@ -7255,6 +8094,11 @@
           <t>Makes the Pokémon eat any held Berry triggered by low HP below 1/2 its max HP.</t>
         </is>
       </c>
+      <c r="O84" t="inlineStr">
+        <is>
+          <t>Come a fruta mais cedo, com HP abaixo da metade.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -7727,13 +8571,43 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Revide</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>REVIDE</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
         </is>
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Depois de ser atingido, o próximo golpe causa 6% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
+        <v>3</v>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K92" t="n">
+        <v>6</v>
+      </c>
+      <c r="L92" t="n">
+        <v>20</v>
       </c>
       <c r="M92" t="n">
         <v>3</v>
@@ -7743,6 +8617,11 @@
           <t>If a Cramorant with Gulp Missile uses Surf or Dive, it catches prey and changes its form depending on its remaining HP.</t>
         </is>
       </c>
+      <c r="O92" t="inlineStr">
+        <is>
+          <t>Captura presas ao usar Surf e as lança quando atingido.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -8087,13 +8966,43 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Defesa leve</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>CASCO</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Golpes causam 4% a 12% menos dano.</t>
+        </is>
+      </c>
+      <c r="I98" t="n">
+        <v>3</v>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K98" t="n">
+        <v>4</v>
+      </c>
+      <c r="L98" t="n">
+        <v>12</v>
       </c>
       <c r="M98" t="n">
         <v>10</v>
@@ -8103,6 +9012,11 @@
           <t>Doubles the Pokémon's weight.</t>
         </is>
       </c>
+      <c r="O98" t="inlineStr">
+        <is>
+          <t>Dobra o peso.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -8117,13 +9031,43 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Cura gradual</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>CURA_GRADUAL</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Cura 3% a 10% do HP máximo.</t>
+        </is>
+      </c>
+      <c r="I99" t="n">
+        <v>3</v>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K99" t="n">
+        <v>3</v>
+      </c>
+      <c r="L99" t="n">
+        <v>10</v>
       </c>
       <c r="M99" t="n">
         <v>5</v>
@@ -8133,6 +9077,11 @@
           <t>The Pokémon may pick up Honey after battle.</t>
         </is>
       </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>Pode achar mel depois da batalha.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -8275,13 +9224,43 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Impulso</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>IMPULSO</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Nas 3 primeiras rodadas, ganha Agilidade, até 4% a 12% no total.</t>
+        </is>
+      </c>
+      <c r="I102" t="n">
+        <v>3</v>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Agilidade</t>
+        </is>
+      </c>
+      <c r="K102" t="n">
+        <v>4</v>
+      </c>
+      <c r="L102" t="n">
+        <v>12</v>
       </c>
       <c r="M102" t="n">
         <v>2</v>
@@ -8291,6 +9270,11 @@
           <t>Causes Morpeko to change its form each turn, alternating between Full Belly Mode and Hangry Mode</t>
         </is>
       </c>
+      <c r="O102" t="inlineStr">
+        <is>
+          <t>Alterna entre duas formas a cada turno.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -8689,13 +9673,43 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Golpe certeiro</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>QUEBRA_GUARDA</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Ignora 6% a 20% da mitigação (Vitalidade) do alvo.</t>
+        </is>
+      </c>
+      <c r="I109" t="n">
+        <v>2</v>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K109" t="n">
+        <v>6</v>
+      </c>
+      <c r="L109" t="n">
+        <v>20</v>
       </c>
       <c r="M109" t="n">
         <v>8</v>
@@ -8705,6 +9719,11 @@
           <t>Doubles the wild encounter rate.</t>
         </is>
       </c>
+      <c r="O109" t="inlineStr">
+        <is>
+          <t>Dobra a chance de encontros selvagens e evita perda de precisão.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -8719,13 +9738,43 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Evasiva</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>EVASIVA</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Esquiva parcial: o golpe causa 4% a 12% menos dano.</t>
+        </is>
+      </c>
+      <c r="I110" t="n">
+        <v>3</v>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>Agilidade</t>
+        </is>
+      </c>
+      <c r="K110" t="n">
+        <v>4</v>
+      </c>
+      <c r="L110" t="n">
+        <v>12</v>
       </c>
       <c r="M110" t="n">
         <v>2</v>
@@ -8735,6 +9784,11 @@
           <t>Takes the appearance of the last conscious party Pokémon upon being sent out until hit by a damaging move.</t>
         </is>
       </c>
+      <c r="O110" t="inlineStr">
+        <is>
+          <t>Disfarça-se como outro Pokémon até ser atingido.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -8813,13 +9867,43 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>Espelho</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>ESPELHO</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Ao receber debuff</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Devolve 6% a 20% do debuff recebido a quem o aplicou.</t>
+        </is>
+      </c>
+      <c r="I112" t="n">
+        <v>2</v>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K112" t="n">
+        <v>6</v>
+      </c>
+      <c r="L112" t="n">
+        <v>20</v>
       </c>
       <c r="M112" t="n">
         <v>1</v>
@@ -8829,6 +9913,11 @@
           <t>Transforms upon entering battle.</t>
         </is>
       </c>
+      <c r="O112" t="inlineStr">
+        <is>
+          <t>Transforma-se no Pokémon rival ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -9493,13 +10582,43 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>Adversidade</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>ADVERSIDADE</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Ao receber debuff</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Ao ter um atributo reduzido, o próximo golpe causa 8% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I123" t="n">
+        <v>2</v>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K123" t="n">
+        <v>8</v>
+      </c>
+      <c r="L123" t="n">
+        <v>20</v>
       </c>
       <c r="M123" t="n">
         <v>12</v>
@@ -9509,6 +10628,11 @@
           <t>Prevents the Pokémon from using its held item in battle.</t>
         </is>
       </c>
+      <c r="O123" t="inlineStr">
+        <is>
+          <t>Não consegue usar o item que segura.</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -9656,13 +10780,43 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>Vantagem ampliada</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>VANTAGEM</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Golpes com vantagem de tipo causam 6% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I126" t="n">
+        <v>2</v>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K126" t="n">
+        <v>6</v>
+      </c>
+      <c r="L126" t="n">
+        <v>20</v>
       </c>
       <c r="M126" t="n">
         <v>4</v>
@@ -9672,6 +10826,11 @@
           <t>Libero changes the Pokémon's type to that of its previously used attack.</t>
         </is>
       </c>
+      <c r="O126" t="inlineStr">
+        <is>
+          <t>Muda de tipo para o do último golpe usado.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -9686,13 +10845,43 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Evasiva</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>EVASIVA</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Esquiva parcial: o golpe causa 4% a 12% menos dano.</t>
+        </is>
+      </c>
+      <c r="I127" t="n">
+        <v>3</v>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Agilidade</t>
+        </is>
+      </c>
+      <c r="K127" t="n">
+        <v>4</v>
+      </c>
+      <c r="L127" t="n">
+        <v>12</v>
       </c>
       <c r="M127" t="n">
         <v>7</v>
@@ -9702,6 +10891,11 @@
           <t>Halves the Pokémon's weight.</t>
         </is>
       </c>
+      <c r="O127" t="inlineStr">
+        <is>
+          <t>Reduz o peso pela metade.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -10237,13 +11431,43 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>Roubo de vida</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>VAMPIRISMO</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Recupera 6% a 15% do dano causado.</t>
+        </is>
+      </c>
+      <c r="I136" t="n">
+        <v>3</v>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K136" t="n">
+        <v>6</v>
+      </c>
+      <c r="L136" t="n">
+        <v>15</v>
       </c>
       <c r="M136" t="n">
         <v>6</v>
@@ -10253,6 +11477,11 @@
           <t>Steals the target's held item when the bearer uses a damaging move.</t>
         </is>
       </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>Rouba o item do alvo ao atingir.</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -10331,13 +11560,47 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Controle</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Intimidação</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>INTIMIDACAO</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Agilidade</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Início da luta</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Reduz Agilidade de todos os rivais em 4% a 12%.</t>
+        </is>
+      </c>
+      <c r="I138" t="n">
+        <v>1</v>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Carisma</t>
+        </is>
+      </c>
+      <c r="K138" t="n">
+        <v>4</v>
+      </c>
+      <c r="L138" t="n">
+        <v>12</v>
       </c>
       <c r="M138" t="n">
         <v>6</v>
@@ -10347,6 +11610,11 @@
           <t>Prevents Steel opponents from fleeing or switching out.</t>
         </is>
       </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>Impede rivais de Aço de fugir ou trocar.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -10627,13 +11895,43 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Vantagem ampliada</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>VANTAGEM</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Golpes com vantagem de tipo causam 6% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I143" t="n">
+        <v>2</v>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K143" t="n">
+        <v>6</v>
+      </c>
+      <c r="L143" t="n">
+        <v>20</v>
       </c>
       <c r="M143" t="n">
         <v>1</v>
@@ -10643,6 +11941,11 @@
           <t>Changes type depending on the terrain.</t>
         </is>
       </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>Muda de tipo conforme o terreno.</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -11243,13 +12546,43 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>Vantagem ampliada</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>VANTAGEM</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H153" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Golpes com vantagem de tipo causam 6% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I153" t="n">
+        <v>2</v>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K153" t="n">
+        <v>6</v>
+      </c>
+      <c r="L153" t="n">
+        <v>20</v>
       </c>
       <c r="M153" t="n">
         <v>1</v>
@@ -11259,6 +12592,11 @@
           <t>Changes Arceus's type and form to match its held Plate.</t>
         </is>
       </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>Muda de tipo conforme a placa que segura.</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -11342,13 +12680,43 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Golpe certeiro</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>QUEBRA_GUARDA</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H155" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Ignora 6% a 20% da mitigação (Vitalidade) do alvo.</t>
+        </is>
+      </c>
+      <c r="I155" t="n">
+        <v>2</v>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K155" t="n">
+        <v>6</v>
+      </c>
+      <c r="L155" t="n">
+        <v>20</v>
       </c>
       <c r="M155" t="n">
         <v>2</v>
@@ -11358,6 +12726,11 @@
           <t>Status moves go last, but are not affected by the opponent's ability.</t>
         </is>
       </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>Golpes de status agem por último, mas ignoram habilidades do alvo.</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -11500,12 +12873,36 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>Anula bônus rivais</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>ANULAR_BONUS</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
         </is>
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
+          <t>Nas 3 primeiras rodadas, anula os bônus de Ambiente e de Aura dos rivais.</t>
+        </is>
+      </c>
+      <c r="I158" t="n">
+        <v>3</v>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>Instinto</t>
         </is>
       </c>
       <c r="M158" t="n">
@@ -11516,6 +12913,11 @@
           <t>Neutralizes abilities of all Pokémon in battle.</t>
         </is>
       </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>Neutraliza as habilidades de todos em campo.</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -11594,13 +12996,47 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>Maestria elemental</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>MAESTRIA_TIPO</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Se o mascote tem o tipo Normal, seus golpes causam 6% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I160" t="n">
+        <v>2</v>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K160" t="n">
+        <v>6</v>
+      </c>
+      <c r="L160" t="n">
+        <v>20</v>
       </c>
       <c r="M160" t="n">
         <v>2</v>
@@ -11610,6 +13046,11 @@
           <t>Makes the Pokémon's moves all act Normal-type.</t>
         </is>
       </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>Todos os seus golpes viram Normais.</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -11688,13 +13129,43 @@
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>Revide</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>REVIDE</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr"/>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Depois de ser atingido, o próximo golpe causa 6% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I162" t="n">
+        <v>3</v>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K162" t="n">
+        <v>6</v>
+      </c>
+      <c r="L162" t="n">
+        <v>20</v>
       </c>
       <c r="M162" t="n">
         <v>1</v>
@@ -11704,6 +13175,11 @@
           <t>Copies stat boosts by the opponent.</t>
         </is>
       </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>Copia os aumentos de atributo do rival.</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -12112,13 +13588,43 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>Roubo de vida</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>VAMPIRISMO</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr"/>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Recupera 6% a 15% do dano causado.</t>
+        </is>
+      </c>
+      <c r="I169" t="n">
+        <v>3</v>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K169" t="n">
+        <v>6</v>
+      </c>
+      <c r="L169" t="n">
+        <v>15</v>
       </c>
       <c r="M169" t="n">
         <v>15</v>
@@ -12128,6 +13634,11 @@
           <t>Steals attacking Pokémon's held items on contact.</t>
         </is>
       </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>Rouba o item de quem o atinge com contato.</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -12142,13 +13653,43 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>Cura gradual</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>CURA_GRADUAL</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr"/>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Cura 3% a 10% do HP máximo.</t>
+        </is>
+      </c>
+      <c r="I170" t="n">
+        <v>3</v>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K170" t="n">
+        <v>3</v>
+      </c>
+      <c r="L170" t="n">
+        <v>10</v>
       </c>
       <c r="M170" t="n">
         <v>26</v>
@@ -12158,6 +13699,11 @@
           <t>Picks up other Pokémon's used and Flung held items.  May also pick up an item after battle.</t>
         </is>
       </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>Pega itens usados ou largados.</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -12640,13 +14186,43 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>Fúria</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>FURIA</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>HP baixo (abaixo de 33%)</t>
         </is>
       </c>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Os golpes causam 6% a 18% mais dano.</t>
+        </is>
+      </c>
+      <c r="I178" t="n">
+        <v>2</v>
+      </c>
+      <c r="J178" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K178" t="n">
+        <v>6</v>
+      </c>
+      <c r="L178" t="n">
+        <v>18</v>
       </c>
       <c r="M178" t="n">
         <v>3</v>
@@ -12656,6 +14232,11 @@
           <t>Transforms 10% or 50% Zygarde into Complete Forme when its HP is below 50%.</t>
         </is>
       </c>
+      <c r="O178" t="inlineStr">
+        <is>
+          <t>Muda de forma com HP abaixo da metade.</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -13000,13 +14581,43 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D184" t="inlineStr">
+        <is>
+          <t>Evasiva</t>
+        </is>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>EVASIVA</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Esquiva parcial: o golpe causa 4% a 12% menos dano.</t>
+        </is>
+      </c>
+      <c r="I184" t="n">
+        <v>3</v>
+      </c>
+      <c r="J184" t="inlineStr">
+        <is>
+          <t>Agilidade</t>
+        </is>
+      </c>
+      <c r="K184" t="n">
+        <v>4</v>
+      </c>
+      <c r="L184" t="n">
+        <v>12</v>
       </c>
       <c r="M184" t="n">
         <v>2</v>
@@ -13016,6 +14627,11 @@
           <t>Ignores moves and abilities that draw in moves.</t>
         </is>
       </c>
+      <c r="O184" t="inlineStr">
+        <is>
+          <t>Ignora golpes e habilidades que atraem ataques.</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -13030,13 +14646,43 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Vantagem ampliada</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>VANTAGEM</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr"/>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Golpes com vantagem de tipo causam 6% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I185" t="n">
+        <v>2</v>
+      </c>
+      <c r="J185" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K185" t="n">
+        <v>6</v>
+      </c>
+      <c r="L185" t="n">
+        <v>20</v>
       </c>
       <c r="M185" t="n">
         <v>8</v>
@@ -13046,6 +14692,11 @@
           <t>Changes the bearer's type to match each move it uses.</t>
         </is>
       </c>
+      <c r="O185" t="inlineStr">
+        <is>
+          <t>Muda de tipo para o de cada golpe usado.</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -13981,13 +15632,43 @@
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Cura gradual</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>CURA_GRADUAL</t>
+        </is>
+      </c>
+      <c r="F200" t="inlineStr"/>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Cura 3% a 10% do HP máximo.</t>
+        </is>
+      </c>
+      <c r="I200" t="n">
+        <v>3</v>
+      </c>
+      <c r="J200" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K200" t="n">
+        <v>3</v>
+      </c>
+      <c r="L200" t="n">
+        <v>10</v>
       </c>
       <c r="M200" t="n">
         <v>5</v>
@@ -13997,6 +15678,11 @@
           <t>Doubles the effect of berries.</t>
         </is>
       </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>Dobra o efeito das frutas.</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -14011,13 +15697,43 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Ataque reforçado</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>PODER_BRUTO</t>
+        </is>
+      </c>
+      <c r="F201" t="inlineStr"/>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Nas duas primeiras ações, o golpe causa 8% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I201" t="n">
+        <v>2</v>
+      </c>
+      <c r="J201" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K201" t="n">
+        <v>8</v>
+      </c>
+      <c r="L201" t="n">
+        <v>20</v>
       </c>
       <c r="M201" t="n">
         <v>18</v>
@@ -14027,6 +15743,11 @@
           <t>Increases damage inflicted to 1.25× against Pokémon of the same gender, but decreases damage to 0.75× against the opposite gender.</t>
         </is>
       </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>Mais dano contra o mesmo gênero e menos contra o oposto.</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -14041,13 +15762,43 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Vantagem ampliada</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>VANTAGEM</t>
+        </is>
+      </c>
+      <c r="F202" t="inlineStr"/>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Golpes com vantagem de tipo causam 6% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I202" t="n">
+        <v>2</v>
+      </c>
+      <c r="J202" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K202" t="n">
+        <v>6</v>
+      </c>
+      <c r="L202" t="n">
+        <v>20</v>
       </c>
       <c r="M202" t="n">
         <v>1</v>
@@ -14057,6 +15808,11 @@
           <t>Changes this Pokémon's type to match its held Memory.</t>
         </is>
       </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>Muda de tipo conforme a memória que segura.</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -14268,13 +16024,43 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Evasiva</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>EVASIVA</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr"/>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Esquiva parcial: o golpe causa 4% a 12% menos dano.</t>
+        </is>
+      </c>
+      <c r="I206" t="n">
+        <v>3</v>
+      </c>
+      <c r="J206" t="inlineStr">
+        <is>
+          <t>Agilidade</t>
+        </is>
+      </c>
+      <c r="K206" t="n">
+        <v>4</v>
+      </c>
+      <c r="L206" t="n">
+        <v>12</v>
       </c>
       <c r="M206" t="n">
         <v>33</v>
@@ -14284,6 +16070,11 @@
           <t>Ensures success fleeing from wild battles.</t>
         </is>
       </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>Foge com certeza de batalhas selvagens.</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -14431,13 +16222,47 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Ambiente</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>AMBIENTE</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>Pedra</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>Início da luta</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Nas 3 primeiras rodadas, aliados do tipo Pedra causam 4% a 12% mais dano.</t>
+        </is>
+      </c>
+      <c r="I209" t="n">
+        <v>3</v>
+      </c>
+      <c r="J209" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K209" t="n">
+        <v>4</v>
+      </c>
+      <c r="L209" t="n">
+        <v>12</v>
       </c>
       <c r="M209" t="n">
         <v>3</v>
@@ -14447,6 +16272,11 @@
           <t>Creates a sandstorm when hit by an attack.</t>
         </is>
       </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>Cria tempestade de areia ao ser atingido.</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -14663,13 +16493,43 @@
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Escamas</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>ESCAMAS</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr"/>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>O primeiro golpe recebido com HP cheio causa 8% a 20% menos dano.</t>
+        </is>
+      </c>
+      <c r="I213" t="n">
+        <v>1</v>
+      </c>
+      <c r="J213" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K213" t="n">
+        <v>8</v>
+      </c>
+      <c r="L213" t="n">
+        <v>20</v>
       </c>
       <c r="M213" t="n">
         <v>2</v>
@@ -14679,6 +16539,11 @@
           <t>Wishiwashi becomes Schooling Form when its HP is 25% or higher.</t>
         </is>
       </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>Forma cardume quando o HP está alto.</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -14757,12 +16622,36 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Anula bônus rivais</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>ANULAR_BONUS</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr"/>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
+          <t>Nas 3 primeiras rodadas, anula os bônus de Ambiente e de Aura dos rivais.</t>
+        </is>
+      </c>
+      <c r="I215" t="n">
+        <v>3</v>
+      </c>
+      <c r="J215" t="inlineStr">
+        <is>
+          <t>Instinto</t>
         </is>
       </c>
       <c r="M215" t="n">
@@ -14773,6 +16662,11 @@
           <t>Nullifies effects of Light Screen, Reflect, and Aurora Veil.</t>
         </is>
       </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>Anula barreiras como Reflect e Light Screen.</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -14856,13 +16750,43 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Golpe feliz</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>GOLPE_FELIZ</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr"/>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>30% de chance de o golpe causar 8% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I217" t="n">
+        <v>3</v>
+      </c>
+      <c r="J217" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K217" t="n">
+        <v>8</v>
+      </c>
+      <c r="L217" t="n">
+        <v>20</v>
       </c>
       <c r="M217" t="n">
         <v>14</v>
@@ -14872,6 +16796,11 @@
           <t>Doubles the chance of moves' extra effects occurring.</t>
         </is>
       </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>Dobra a chance dos efeitos extras dos golpes.</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -14950,13 +16879,47 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Controle</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>Intimidação</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>INTIMIDACAO</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>Agilidade</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>Início da luta</t>
         </is>
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Reduz Agilidade de todos os rivais em 4% a 12%.</t>
+        </is>
+      </c>
+      <c r="I219" t="n">
+        <v>1</v>
+      </c>
+      <c r="J219" t="inlineStr">
+        <is>
+          <t>Carisma</t>
+        </is>
+      </c>
+      <c r="K219" t="n">
+        <v>4</v>
+      </c>
+      <c r="L219" t="n">
+        <v>12</v>
       </c>
       <c r="M219" t="n">
         <v>6</v>
@@ -14966,6 +16929,11 @@
           <t>Prevents opponents from fleeing or switching out.</t>
         </is>
       </c>
+      <c r="O219" t="inlineStr">
+        <is>
+          <t>Impede os rivais de fugir ou trocar.</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -15310,13 +17278,43 @@
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>Escamas</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>ESCAMAS</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr"/>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
         </is>
       </c>
       <c r="H225" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>O primeiro golpe recebido com HP cheio causa 8% a 20% menos dano.</t>
+        </is>
+      </c>
+      <c r="I225" t="n">
+        <v>1</v>
+      </c>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K225" t="n">
+        <v>8</v>
+      </c>
+      <c r="L225" t="n">
+        <v>20</v>
       </c>
       <c r="M225" t="n">
         <v>14</v>
@@ -15326,6 +17324,11 @@
           <t>Transforms this Minior between Core Form and Meteor Form.  Prevents major status ailments and drowsiness while in Meteor Form.</t>
         </is>
       </c>
+      <c r="O225" t="inlineStr">
+        <is>
+          <t>Muda de forma quando o HP cai abaixo da metade.</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -15340,13 +17343,43 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Adversidade</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>ADVERSIDADE</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr"/>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>Ao receber debuff</t>
         </is>
       </c>
       <c r="H226" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Ao ter um atributo reduzido, o próximo golpe causa 8% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I226" t="n">
+        <v>2</v>
+      </c>
+      <c r="J226" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K226" t="n">
+        <v>8</v>
+      </c>
+      <c r="L226" t="n">
+        <v>20</v>
       </c>
       <c r="M226" t="n">
         <v>5</v>
@@ -15356,6 +17389,11 @@
           <t>Doubles the Pokémon's stat modifiers.  These doubled modifiers are still capped at -6 or 6 stages.</t>
         </is>
       </c>
+      <c r="O226" t="inlineStr">
+        <is>
+          <t>Dobra as mudanças de atributo.</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -15434,13 +17472,43 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Aquecimento</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>AQUECIMENTO</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr"/>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
         </is>
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Nas 2 primeiras rodadas recebe 6% a 20% menos dano; depois, seus 3 golpes seguintes causam 6% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I228" t="n">
+        <v>3</v>
+      </c>
+      <c r="J228" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K228" t="n">
+        <v>6</v>
+      </c>
+      <c r="L228" t="n">
+        <v>20</v>
       </c>
       <c r="M228" t="n">
         <v>2</v>
@@ -15450,6 +17518,11 @@
           <t>Halves Attack and Speed for five turns upon entering battle.</t>
         </is>
       </c>
+      <c r="O228" t="inlineStr">
+        <is>
+          <t>Corta Ataque e Velocidade pela metade nos primeiros 5 turnos.</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -16173,13 +18246,43 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Último a agir</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>ULTIMO</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr"/>
+      <c r="G240" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H240" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Ao agir depois dos aliados na rodada, o golpe causa 6% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I240" t="n">
+        <v>2</v>
+      </c>
+      <c r="J240" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K240" t="n">
+        <v>6</v>
+      </c>
+      <c r="L240" t="n">
+        <v>20</v>
       </c>
       <c r="M240" t="n">
         <v>1</v>
@@ -16189,6 +18292,11 @@
           <t>Makes the Pokémon move last within its move's priority bracket.</t>
         </is>
       </c>
+      <c r="O240" t="inlineStr">
+        <is>
+          <t>Sempre age por último dentro da prioridade.</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -16203,13 +18311,43 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Golpe certeiro</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>QUEBRA_GUARDA</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr"/>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Ignora 6% a 20% da mitigação (Vitalidade) do alvo.</t>
+        </is>
+      </c>
+      <c r="I241" t="n">
+        <v>2</v>
+      </c>
+      <c r="J241" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K241" t="n">
+        <v>6</v>
+      </c>
+      <c r="L241" t="n">
+        <v>20</v>
       </c>
       <c r="M241" t="n">
         <v>4</v>
@@ -16219,6 +18357,11 @@
           <t>Ignores moves and abilities that draw in moves.</t>
         </is>
       </c>
+      <c r="O241" t="inlineStr">
+        <is>
+          <t>Ignora golpes e habilidades que atraem ataques.</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -16297,13 +18440,43 @@
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Ataque reforçado</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>PODER_BRUTO</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr"/>
+      <c r="G243" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Nas duas primeiras ações, o golpe causa 8% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I243" t="n">
+        <v>2</v>
+      </c>
+      <c r="J243" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K243" t="n">
+        <v>8</v>
+      </c>
+      <c r="L243" t="n">
+        <v>20</v>
       </c>
       <c r="M243" t="n">
         <v>2</v>
@@ -16313,6 +18486,11 @@
           <t>Changes Aegislash to Blade Forme before using a damaging move, or Shield Forme before using King’s Shield.</t>
         </is>
       </c>
+      <c r="O243" t="inlineStr">
+        <is>
+          <t>Muda de forma conforme usa ataques ou defesa.</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -16396,13 +18574,43 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Revide</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>REVIDE</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr"/>
+      <c r="G245" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Depois de ser atingido, o próximo golpe causa 6% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I245" t="n">
+        <v>3</v>
+      </c>
+      <c r="J245" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K245" t="n">
+        <v>6</v>
+      </c>
+      <c r="L245" t="n">
+        <v>20</v>
       </c>
       <c r="M245" t="n">
         <v>15</v>
@@ -16412,6 +18620,11 @@
           <t>Raises Speed one stage upon flinching.</t>
         </is>
       </c>
+      <c r="O245" t="inlineStr">
+        <is>
+          <t>Velocidade sobe ao recuar (flinch).</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
@@ -16697,13 +18910,43 @@
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Resistência a debuff</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>CORPO_LIMPO</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr"/>
+      <c r="G250" t="inlineStr">
+        <is>
+          <t>Ao receber debuff</t>
         </is>
       </c>
       <c r="H250" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Debuffs recebidos ficam 8% a 20% menores.</t>
+        </is>
+      </c>
+      <c r="I250" t="n">
+        <v>3</v>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K250" t="n">
+        <v>8</v>
+      </c>
+      <c r="L250" t="n">
+        <v>20</v>
       </c>
       <c r="M250" t="n">
         <v>10</v>
@@ -16713,6 +18956,11 @@
           <t>Prevents a held item from being removed by other Pokémon.</t>
         </is>
       </c>
+      <c r="O250" t="inlineStr">
+        <is>
+          <t>Impede que lhe roubem o item.</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -16923,13 +19171,43 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Resistência a debuff</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>CORPO_LIMPO</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr"/>
+      <c r="G254" t="inlineStr">
+        <is>
+          <t>Ao receber debuff</t>
         </is>
       </c>
       <c r="H254" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Debuffs recebidos ficam 8% a 20% menores.</t>
+        </is>
+      </c>
+      <c r="I254" t="n">
+        <v>3</v>
+      </c>
+      <c r="J254" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K254" t="n">
+        <v>8</v>
+      </c>
+      <c r="L254" t="n">
+        <v>20</v>
       </c>
       <c r="M254" t="n">
         <v>5</v>
@@ -16939,6 +19217,11 @@
           <t>Prevents being forced out of battle by other Pokémon's moves.</t>
         </is>
       </c>
+      <c r="O254" t="inlineStr">
+        <is>
+          <t>Impede ser forçado a sair de campo.</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
@@ -17746,13 +20029,43 @@
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>Guarda de aliados</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>GUARDA</t>
+        </is>
+      </c>
+      <c r="F267" t="inlineStr"/>
+      <c r="G267" t="inlineStr">
+        <is>
+          <t>Ao proteger</t>
         </is>
       </c>
       <c r="H267" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Quando o Guardião protege um aliado, o golpe causa 6% a 20% menos dano.</t>
+        </is>
+      </c>
+      <c r="I267" t="n">
+        <v>3</v>
+      </c>
+      <c r="J267" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K267" t="n">
+        <v>6</v>
+      </c>
+      <c r="L267" t="n">
+        <v>20</v>
       </c>
       <c r="M267" t="n">
         <v>28</v>
@@ -17762,6 +20075,11 @@
           <t>Protects against friendly Pokémon's damaging moves.</t>
         </is>
       </c>
+      <c r="O267" t="inlineStr">
+        <is>
+          <t>Evita golpes dos aliados.</t>
+        </is>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
@@ -17840,13 +20158,43 @@
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>Armadura de tipos</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>ARMADURA</t>
+        </is>
+      </c>
+      <c r="F269" t="inlineStr"/>
+      <c r="G269" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
         </is>
       </c>
       <c r="H269" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Golpes com vantagem de tipo contra este mascote causam 6% a 20% menos dano.</t>
+        </is>
+      </c>
+      <c r="I269" t="n">
+        <v>3</v>
+      </c>
+      <c r="J269" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K269" t="n">
+        <v>6</v>
+      </c>
+      <c r="L269" t="n">
+        <v>20</v>
       </c>
       <c r="M269" t="n">
         <v>1</v>
@@ -17856,6 +20204,11 @@
           <t xml:space="preserve">When Terapagos enters the battle, it turns into its Terastal Form until the end of the battle. </t>
         </is>
       </c>
+      <c r="O269" t="inlineStr">
+        <is>
+          <t>Assume a forma Terastal ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -17870,12 +20223,36 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>Anula bônus rivais</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>ANULAR_BONUS</t>
+        </is>
+      </c>
+      <c r="F270" t="inlineStr"/>
+      <c r="G270" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
         </is>
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
+          <t>Nas 3 primeiras rodadas, anula os bônus de Ambiente e de Aura dos rivais.</t>
+        </is>
+      </c>
+      <c r="I270" t="n">
+        <v>3</v>
+      </c>
+      <c r="J270" t="inlineStr">
+        <is>
+          <t>Instinto</t>
         </is>
       </c>
       <c r="M270" t="n">
@@ -17886,6 +20263,11 @@
           <t xml:space="preserve">As soon as Terapagos assumes its Stellar Form, it will immediately neutralize weather and terrain effects. </t>
         </is>
       </c>
+      <c r="O270" t="inlineStr">
+        <is>
+          <t>Neutraliza clima e terreno ao assumir a forma Estelar.</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -18496,13 +20878,43 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Espelho</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>ESPELHO</t>
+        </is>
+      </c>
+      <c r="F280" t="inlineStr"/>
+      <c r="G280" t="inlineStr">
+        <is>
+          <t>Ao receber debuff</t>
         </is>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Devolve 6% a 20% do debuff recebido a quem o aplicou.</t>
+        </is>
+      </c>
+      <c r="I280" t="n">
+        <v>2</v>
+      </c>
+      <c r="J280" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K280" t="n">
+        <v>6</v>
+      </c>
+      <c r="L280" t="n">
+        <v>20</v>
       </c>
       <c r="M280" t="n">
         <v>8</v>
@@ -18512,6 +20924,11 @@
           <t>Copies an opponent's ability upon entering battle.</t>
         </is>
       </c>
+      <c r="O280" t="inlineStr">
+        <is>
+          <t>Copia a habilidade do rival ao entrar.</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -18659,13 +21076,43 @@
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>Aquecimento</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>AQUECIMENTO</t>
+        </is>
+      </c>
+      <c r="F283" t="inlineStr"/>
+      <c r="G283" t="inlineStr">
+        <is>
+          <t>Início da rodada</t>
         </is>
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Nas 2 primeiras rodadas recebe 6% a 20% menos dano; depois, seus 3 golpes seguintes causam 6% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I283" t="n">
+        <v>3</v>
+      </c>
+      <c r="J283" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K283" t="n">
+        <v>6</v>
+      </c>
+      <c r="L283" t="n">
+        <v>20</v>
       </c>
       <c r="M283" t="n">
         <v>3</v>
@@ -18675,6 +21122,11 @@
           <t>Skips every second turn.</t>
         </is>
       </c>
+      <c r="O283" t="inlineStr">
+        <is>
+          <t>Só age em turnos alternados.</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -20137,13 +22589,43 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>Fúria</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>FURIA</t>
+        </is>
+      </c>
+      <c r="F306" t="inlineStr"/>
+      <c r="G306" t="inlineStr">
+        <is>
+          <t>HP baixo (abaixo de 33%)</t>
         </is>
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Os golpes causam 6% a 18% mais dano.</t>
+        </is>
+      </c>
+      <c r="I306" t="n">
+        <v>2</v>
+      </c>
+      <c r="J306" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K306" t="n">
+        <v>6</v>
+      </c>
+      <c r="L306" t="n">
+        <v>18</v>
       </c>
       <c r="M306" t="n">
         <v>4</v>
@@ -20153,6 +22635,11 @@
           <t>Changes Darmanitan's form after each turn depending on its HP: Zen Mode below 50% max HP, and Standard Mode otherwise.</t>
         </is>
       </c>
+      <c r="O306" t="inlineStr">
+        <is>
+          <t>Muda de forma com HP abaixo da metade.</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
@@ -20167,13 +22654,43 @@
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>Sem efeito</t>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Vingança</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>VINGANCA</t>
+        </is>
+      </c>
+      <c r="F307" t="inlineStr"/>
+      <c r="G307" t="inlineStr">
+        <is>
+          <t>Aliado cai</t>
         </is>
       </c>
       <c r="H307" t="inlineStr">
         <is>
-          <t>Sem efeito em combate nesta versão.</t>
-        </is>
+          <t>Quando um aliado cai, o próximo golpe causa 8% a 20% mais dano.</t>
+        </is>
+      </c>
+      <c r="I307" t="n">
+        <v>1</v>
+      </c>
+      <c r="J307" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="K307" t="n">
+        <v>8</v>
+      </c>
+      <c r="L307" t="n">
+        <v>20</v>
       </c>
       <c r="M307" t="n">
         <v>2</v>
@@ -20181,6 +22698,11 @@
       <c r="N307" t="inlineStr">
         <is>
           <t>Transforms into its Hero Form when switching out.</t>
+        </is>
+      </c>
+      <c r="O307" t="inlineStr">
+        <is>
+          <t>Assume a forma Heroica ao sair de campo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: explica Ambiente, Aura e Aquecimento nas descricoes, na aba Habilidades e no manual
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/habilidades-passivas-mascotes.xlsx
+++ b/docs/habilidades-passivas-mascotes.xlsx
@@ -2227,7 +2227,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Aliados do tipo {T} causam {rng} mais dano.</t>
+          <t>Aura da habilidade: enquanto o mascote estiver em campo, aliados do tipo {T} causam {rng} mais dano nos golpes (2 vezes por luta).</t>
         </is>
       </c>
       <c r="F44" t="n">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo {T} causam {rng} mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo {T} causam {rng} mais dano.</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, anula os bônus de Ambiente e de Aura dos rivais.</t>
+          <t>Nas 3 primeiras rodadas, os rivais ficam sem os bônus de dano de Ambiente (clima/terreno criado por habilidades como Drought ou Drizzle) e de Aura (como Fairy Aura ou Dark Aura).</t>
         </is>
       </c>
       <c r="F48" t="n">
@@ -2461,7 +2461,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Nas 2 primeiras rodadas recebe {rng} menos dano; depois, seus 3 golpes seguintes causam {rng} mais dano.</t>
+          <t>Nas 2 primeiras rodadas, recebe {rng} menos dano. A partir da 3ª rodada, os 3 golpes seguintes que ele dá causam {rng} mais dano. Nunca recebe mais dano por causa disto.</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -2892,7 +2892,6 @@
           <t>ANULAR_BONUS</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Início da rodada</t>
@@ -2900,7 +2899,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, anula os bônus de Ambiente e de Aura dos rivais.</t>
+          <t>Nas 3 primeiras rodadas, os rivais ficam sem os bônus de dano de Ambiente (clima/terreno criado por habilidades como Drought ou Drizzle) e de Aura (como Fairy Aura ou Dark Aura).</t>
         </is>
       </c>
       <c r="I5" t="n">
@@ -3143,7 +3142,6 @@
           <t>ARMADURA</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>Ao ser atingido</t>
@@ -3538,7 +3536,6 @@
           <t>ANULAR_BONUS</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>Início da rodada</t>
@@ -3546,7 +3543,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, anula os bônus de Ambiente e de Aura dos rivais.</t>
+          <t>Nas 3 primeiras rodadas, os rivais ficam sem os bônus de dano de Ambiente (clima/terreno criado por habilidades como Drought ou Drizzle) e de Aura (como Fairy Aura ou Dark Aura).</t>
         </is>
       </c>
       <c r="I15" t="n">
@@ -3661,7 +3658,6 @@
           <t>PESADELO</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>Início da rodada</t>
@@ -3726,7 +3722,6 @@
           <t>CURA_GRADUAL</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr">
         <is>
           <t>Início da rodada</t>
@@ -4633,7 +4628,6 @@
           <t>ANULAR_BONUS</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>Início da rodada</t>
@@ -4641,7 +4635,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, anula os bônus de Ambiente e de Aura dos rivais.</t>
+          <t>Nas 3 primeiras rodadas, os rivais ficam sem os bônus de dano de Ambiente (clima/terreno criado por habilidades como Drought ou Drizzle) e de Aura (como Fairy Aura ou Dark Aura).</t>
         </is>
       </c>
       <c r="I32" t="n">
@@ -4692,7 +4686,6 @@
           <t>CASCO</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>Ao ser atingido</t>
@@ -4757,7 +4750,6 @@
           <t>CORPO_LIMPO</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>Ao receber debuff</t>
@@ -4822,7 +4814,6 @@
           <t>REFORCO</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
           <t>Ao aplicar buff</t>
@@ -5015,7 +5006,6 @@
           <t>ADVERSIDADE</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr"/>
       <c r="G38" t="inlineStr">
         <is>
           <t>Ao receber debuff</t>
@@ -5484,7 +5474,6 @@
           <t>IMUNE_INDIRETO</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr"/>
       <c r="G45" t="inlineStr">
         <is>
           <t>Passivo</t>
@@ -5543,7 +5532,6 @@
           <t>GOLPE_DUPLO</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr"/>
       <c r="G46" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -5620,7 +5608,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Aliados do tipo Sombrio causam 4% a 12% mais dano.</t>
+          <t>Aura da habilidade: enquanto o mascote estiver em campo, aliados do tipo Sombrio causam 4% a 12% mais dano nos golpes (2 vezes por luta).</t>
         </is>
       </c>
       <c r="I47" t="n">
@@ -5810,7 +5798,6 @@
           <t>FURIA</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr">
         <is>
           <t>HP baixo (abaixo de 33%)</t>
@@ -5951,7 +5938,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Voador causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Voador causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I52" t="n">
@@ -6020,7 +6007,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Fogo causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Fogo causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I53" t="n">
@@ -6355,7 +6342,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Água causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Água causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I58" t="n">
@@ -6424,7 +6411,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Fogo causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Fogo causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I59" t="n">
@@ -6545,7 +6532,6 @@
           <t>PURIFICACAO</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr">
         <is>
           <t>Ao remover debuff</t>
@@ -6829,7 +6815,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Elétrico causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Elétrico causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I65" t="n">
@@ -7026,7 +7012,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Aliados do tipo Fada causam 4% a 12% mais dano.</t>
+          <t>Aura da habilidade: enquanto o mascote estiver em campo, aliados do tipo Fada causam 4% a 12% mais dano nos golpes (2 vezes por luta).</t>
         </is>
       </c>
       <c r="I68" t="n">
@@ -7610,7 +7596,6 @@
           <t>VANTAGEM</t>
         </is>
       </c>
-      <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -7675,7 +7660,6 @@
           <t>ANALISE</t>
         </is>
       </c>
-      <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
           <t>Início da luta</t>
@@ -7804,7 +7788,6 @@
           <t>ANALISE</t>
         </is>
       </c>
-      <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
           <t>Início da luta</t>
@@ -8061,7 +8044,6 @@
           <t>REGENERACAO</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
           <t>HP baixo (abaixo de 50%)</t>
@@ -8399,7 +8381,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Planta causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Planta causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I89" t="n">
@@ -8584,7 +8566,6 @@
           <t>REVIDE</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr"/>
       <c r="G92" t="inlineStr">
         <is>
           <t>Ao ser atingido</t>
@@ -8725,7 +8706,7 @@
       </c>
       <c r="H94" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Elétrico causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Elétrico causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I94" t="n">
@@ -8979,7 +8960,6 @@
           <t>CASCO</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr"/>
       <c r="G98" t="inlineStr">
         <is>
           <t>Ao ser atingido</t>
@@ -9044,7 +9024,6 @@
           <t>CURA_GRADUAL</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr"/>
       <c r="G99" t="inlineStr">
         <is>
           <t>Início da rodada</t>
@@ -9237,7 +9216,6 @@
           <t>IMPULSO</t>
         </is>
       </c>
-      <c r="F102" t="inlineStr"/>
       <c r="G102" t="inlineStr">
         <is>
           <t>Início da rodada</t>
@@ -9686,7 +9664,6 @@
           <t>QUEBRA_GUARDA</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr"/>
       <c r="G109" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -9751,7 +9728,6 @@
           <t>EVASIVA</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr"/>
       <c r="G110" t="inlineStr">
         <is>
           <t>Ao ser atingido</t>
@@ -9880,7 +9856,6 @@
           <t>ESPELHO</t>
         </is>
       </c>
-      <c r="F112" t="inlineStr"/>
       <c r="G112" t="inlineStr">
         <is>
           <t>Ao receber debuff</t>
@@ -10595,7 +10570,6 @@
           <t>ADVERSIDADE</t>
         </is>
       </c>
-      <c r="F123" t="inlineStr"/>
       <c r="G123" t="inlineStr">
         <is>
           <t>Ao receber debuff</t>
@@ -10793,7 +10767,6 @@
           <t>VANTAGEM</t>
         </is>
       </c>
-      <c r="F126" t="inlineStr"/>
       <c r="G126" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -10858,7 +10831,6 @@
           <t>EVASIVA</t>
         </is>
       </c>
-      <c r="F127" t="inlineStr"/>
       <c r="G127" t="inlineStr">
         <is>
           <t>Ao ser atingido</t>
@@ -11444,7 +11416,6 @@
           <t>VAMPIRISMO</t>
         </is>
       </c>
-      <c r="F136" t="inlineStr"/>
       <c r="G136" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -11787,7 +11758,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Fogo causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Fogo causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I141" t="n">
@@ -11908,7 +11879,6 @@
           <t>VANTAGEM</t>
         </is>
       </c>
-      <c r="F143" t="inlineStr"/>
       <c r="G143" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -12177,7 +12147,7 @@
       </c>
       <c r="H147" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Fada causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Fada causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I147" t="n">
@@ -12559,7 +12529,6 @@
           <t>VANTAGEM</t>
         </is>
       </c>
-      <c r="F153" t="inlineStr"/>
       <c r="G153" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -12693,7 +12662,6 @@
           <t>QUEBRA_GUARDA</t>
         </is>
       </c>
-      <c r="F155" t="inlineStr"/>
       <c r="G155" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -12886,7 +12854,6 @@
           <t>ANULAR_BONUS</t>
         </is>
       </c>
-      <c r="F158" t="inlineStr"/>
       <c r="G158" t="inlineStr">
         <is>
           <t>Início da rodada</t>
@@ -12894,7 +12861,7 @@
       </c>
       <c r="H158" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, anula os bônus de Ambiente e de Aura dos rivais.</t>
+          <t>Nas 3 primeiras rodadas, os rivais ficam sem os bônus de dano de Ambiente (clima/terreno criado por habilidades como Drought ou Drizzle) e de Aura (como Fairy Aura ou Dark Aura).</t>
         </is>
       </c>
       <c r="I158" t="n">
@@ -13142,7 +13109,6 @@
           <t>REVIDE</t>
         </is>
       </c>
-      <c r="F162" t="inlineStr"/>
       <c r="G162" t="inlineStr">
         <is>
           <t>Ao ser atingido</t>
@@ -13219,7 +13185,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Fogo causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Fogo causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I163" t="n">
@@ -13601,7 +13567,6 @@
           <t>VAMPIRISMO</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr"/>
       <c r="G169" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -13666,7 +13631,6 @@
           <t>CURA_GRADUAL</t>
         </is>
       </c>
-      <c r="F170" t="inlineStr"/>
       <c r="G170" t="inlineStr">
         <is>
           <t>Início da rodada</t>
@@ -14199,7 +14163,6 @@
           <t>FURIA</t>
         </is>
       </c>
-      <c r="F178" t="inlineStr"/>
       <c r="G178" t="inlineStr">
         <is>
           <t>HP baixo (abaixo de 33%)</t>
@@ -14473,7 +14436,7 @@
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Água causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Água causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I182" t="n">
@@ -14594,7 +14557,6 @@
           <t>EVASIVA</t>
         </is>
       </c>
-      <c r="F184" t="inlineStr"/>
       <c r="G184" t="inlineStr">
         <is>
           <t>Ao ser atingido</t>
@@ -14659,7 +14621,6 @@
           <t>VANTAGEM</t>
         </is>
       </c>
-      <c r="F185" t="inlineStr"/>
       <c r="G185" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -14800,7 +14761,7 @@
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Psíquico causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Psíquico causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I187" t="n">
@@ -15645,7 +15606,6 @@
           <t>CURA_GRADUAL</t>
         </is>
       </c>
-      <c r="F200" t="inlineStr"/>
       <c r="G200" t="inlineStr">
         <is>
           <t>Início da rodada</t>
@@ -15710,7 +15670,6 @@
           <t>PODER_BRUTO</t>
         </is>
       </c>
-      <c r="F201" t="inlineStr"/>
       <c r="G201" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -15775,7 +15734,6 @@
           <t>VANTAGEM</t>
         </is>
       </c>
-      <c r="F202" t="inlineStr"/>
       <c r="G202" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -16037,7 +15995,6 @@
           <t>EVASIVA</t>
         </is>
       </c>
-      <c r="F206" t="inlineStr"/>
       <c r="G206" t="inlineStr">
         <is>
           <t>Ao ser atingido</t>
@@ -16247,7 +16204,7 @@
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Pedra causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Pedra causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I209" t="n">
@@ -16316,7 +16273,7 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Pedra causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Pedra causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I210" t="n">
@@ -16506,7 +16463,6 @@
           <t>ESCAMAS</t>
         </is>
       </c>
-      <c r="F213" t="inlineStr"/>
       <c r="G213" t="inlineStr">
         <is>
           <t>Ao ser atingido</t>
@@ -16635,7 +16591,6 @@
           <t>ANULAR_BONUS</t>
         </is>
       </c>
-      <c r="F215" t="inlineStr"/>
       <c r="G215" t="inlineStr">
         <is>
           <t>Início da rodada</t>
@@ -16643,7 +16598,7 @@
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, anula os bônus de Ambiente e de Aura dos rivais.</t>
+          <t>Nas 3 primeiras rodadas, os rivais ficam sem os bônus de dano de Ambiente (clima/terreno criado por habilidades como Drought ou Drizzle) e de Aura (como Fairy Aura ou Dark Aura).</t>
         </is>
       </c>
       <c r="I215" t="n">
@@ -16706,7 +16661,7 @@
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Planta causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Planta causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I216" t="n">
@@ -16763,7 +16718,6 @@
           <t>GOLPE_FELIZ</t>
         </is>
       </c>
-      <c r="F217" t="inlineStr"/>
       <c r="G217" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -17291,7 +17245,6 @@
           <t>ESCAMAS</t>
         </is>
       </c>
-      <c r="F225" t="inlineStr"/>
       <c r="G225" t="inlineStr">
         <is>
           <t>Ao ser atingido</t>
@@ -17356,7 +17309,6 @@
           <t>ADVERSIDADE</t>
         </is>
       </c>
-      <c r="F226" t="inlineStr"/>
       <c r="G226" t="inlineStr">
         <is>
           <t>Ao receber debuff</t>
@@ -17485,7 +17437,6 @@
           <t>AQUECIMENTO</t>
         </is>
       </c>
-      <c r="F228" t="inlineStr"/>
       <c r="G228" t="inlineStr">
         <is>
           <t>Início da rodada</t>
@@ -17493,7 +17444,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>Nas 2 primeiras rodadas recebe 6% a 20% menos dano; depois, seus 3 golpes seguintes causam 6% a 20% mais dano.</t>
+          <t>Nas 2 primeiras rodadas, recebe 6% a 20% menos dano. A partir da 3ª rodada, os 3 golpes seguintes que ele dá causam 6% a 20% mais dano. Nunca recebe mais dano por causa disto.</t>
         </is>
       </c>
       <c r="I228" t="n">
@@ -17754,7 +17705,7 @@
       </c>
       <c r="H232" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, aliados do tipo Gelo causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Gelo causam 4% a 12% mais dano.</t>
         </is>
       </c>
       <c r="I232" t="n">
@@ -18259,7 +18210,6 @@
           <t>ULTIMO</t>
         </is>
       </c>
-      <c r="F240" t="inlineStr"/>
       <c r="G240" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -18324,7 +18274,6 @@
           <t>QUEBRA_GUARDA</t>
         </is>
       </c>
-      <c r="F241" t="inlineStr"/>
       <c r="G241" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -18453,7 +18402,6 @@
           <t>PODER_BRUTO</t>
         </is>
       </c>
-      <c r="F243" t="inlineStr"/>
       <c r="G243" t="inlineStr">
         <is>
           <t>Ao atacar</t>
@@ -18587,7 +18535,6 @@
           <t>REVIDE</t>
         </is>
       </c>
-      <c r="F245" t="inlineStr"/>
       <c r="G245" t="inlineStr">
         <is>
           <t>Ao ser atingido</t>
@@ -18797,7 +18744,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>Aliados do tipo Aço causam 4% a 12% mais dano.</t>
+          <t>Aura da habilidade: enquanto o mascote estiver em campo, aliados do tipo Aço causam 4% a 12% mais dano nos golpes (2 vezes por luta).</t>
         </is>
       </c>
       <c r="I248" t="n">
@@ -18923,7 +18870,6 @@
           <t>CORPO_LIMPO</t>
         </is>
       </c>
-      <c r="F250" t="inlineStr"/>
       <c r="G250" t="inlineStr">
         <is>
           <t>Ao receber debuff</t>
@@ -19184,7 +19130,6 @@
           <t>CORPO_LIMPO</t>
         </is>
       </c>
-      <c r="F254" t="inlineStr"/>
       <c r="G254" t="inlineStr">
         <is>
           <t>Ao receber debuff</t>
@@ -20042,7 +19987,6 @@
           <t>GUARDA</t>
         </is>
       </c>
-      <c r="F267" t="inlineStr"/>
       <c r="G267" t="inlineStr">
         <is>
           <t>Ao proteger</t>
@@ -20171,7 +20115,6 @@
           <t>ARMADURA</t>
         </is>
       </c>
-      <c r="F269" t="inlineStr"/>
       <c r="G269" t="inlineStr">
         <is>
           <t>Ao ser atingido</t>
@@ -20236,7 +20179,6 @@
           <t>ANULAR_BONUS</t>
         </is>
       </c>
-      <c r="F270" t="inlineStr"/>
       <c r="G270" t="inlineStr">
         <is>
           <t>Início da rodada</t>
@@ -20244,7 +20186,7 @@
       </c>
       <c r="H270" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, anula os bônus de Ambiente e de Aura dos rivais.</t>
+          <t>Nas 3 primeiras rodadas, os rivais ficam sem os bônus de dano de Ambiente (clima/terreno criado por habilidades como Drought ou Drizzle) e de Aura (como Fairy Aura ou Dark Aura).</t>
         </is>
       </c>
       <c r="I270" t="n">
@@ -20891,7 +20833,6 @@
           <t>ESPELHO</t>
         </is>
       </c>
-      <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
           <t>Ao receber debuff</t>
@@ -21089,7 +21030,6 @@
           <t>AQUECIMENTO</t>
         </is>
       </c>
-      <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
           <t>Início da rodada</t>
@@ -21097,7 +21037,7 @@
       </c>
       <c r="H283" t="inlineStr">
         <is>
-          <t>Nas 2 primeiras rodadas recebe 6% a 20% menos dano; depois, seus 3 golpes seguintes causam 6% a 20% mais dano.</t>
+          <t>Nas 2 primeiras rodadas, recebe 6% a 20% menos dano. A partir da 3ª rodada, os 3 golpes seguintes que ele dá causam 6% a 20% mais dano. Nunca recebe mais dano por causa disto.</t>
         </is>
       </c>
       <c r="I283" t="n">
@@ -22602,7 +22542,6 @@
           <t>FURIA</t>
         </is>
       </c>
-      <c r="F306" t="inlineStr"/>
       <c r="G306" t="inlineStr">
         <is>
           <t>HP baixo (abaixo de 33%)</t>
@@ -22667,7 +22606,6 @@
           <t>VINGANCA</t>
         </is>
       </c>
-      <c r="F307" t="inlineStr"/>
       <c r="G307" t="inlineStr">
         <is>
           <t>Aliado cai</t>

</xml_diff>

<commit_message>
fix(habilidades): Resistência resiste a golpe fatal em qualquer HP
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/habilidades-passivas-mascotes.xlsx
+++ b/docs/habilidades-passivas-mascotes.xlsx
@@ -2350,7 +2350,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Uma vez por luta, sobrevive a um golpe fatal com 1 HP se estiver com HP cheio.</t>
+          <t>Uma vez por luta, resiste a um golpe fatal e fica com 1 HP.</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -19079,7 +19079,7 @@
       </c>
       <c r="H253" t="inlineStr">
         <is>
-          <t>Uma vez por luta, sobrevive a um golpe fatal com 1 HP se estiver com HP cheio.</t>
+          <t>Uma vez por luta, resiste a um golpe fatal e fica com 1 HP.</t>
         </is>
       </c>
       <c r="I253" t="n">

</xml_diff>

<commit_message>
feat(habilidades): sistema de estados alterados (queimado, envenenado, paralisado, dormindo, confuso, congelado, maldito) e efeitos sugeridos pelos GMs
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/habilidades-passivas-mascotes.xlsx
+++ b/docs/habilidades-passivas-mascotes.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>No início da rodada, reduz em {rng} o maior debuff do próprio mascote.</t>
+          <t>No início da rodada, reduz em {rng} o maior debuff do próprio mascote e remove o estado alterado que ele tiver (queimado, envenenado, paralisado, dormindo, confuso ou congelado).</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>No início da rodada, reduz em {rng} o maior debuff de um aliado.</t>
+          <t>No início da rodada, reduz em {rng} o maior debuff de um aliado e remove o estado alterado que ele tiver (queimado, envenenado, paralisado, dormindo, confuso ou congelado).</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -2461,7 +2461,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Nas 2 primeiras rodadas, recebe {rng} menos dano. A partir da 3ª rodada, os 3 golpes seguintes que ele dá causam {rng} mais dano. Nunca recebe mais dano por causa disto.</t>
+          <t>Nas 2 primeiras rodadas recebe de 10% a 15% menos dano (cresce com a Vitalidade). A partir da 3ª rodada, os 3 golpes seguintes que ele dá causam {rng} mais dano. Nunca recebe mais dano por causa disto.</t>
         </is>
       </c>
       <c r="F50" t="n">
@@ -2473,7 +2473,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="I50" t="n">
         <v>20</v>
@@ -2558,6 +2558,1142 @@
         <v>6</v>
       </c>
       <c r="I52" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>ESTADO_CONTATO</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Contágio</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Controle</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Tem {rng} de chance de deixar o atacante {T} (um estado por vez).</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>3</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>6</v>
+      </c>
+      <c r="I53" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>ESTADO_TOQUE</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Toque de estado</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Controle</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Tem {rng} de chance de deixar o alvo {T} ao atacar (um estado por vez).</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>3</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>6</v>
+      </c>
+      <c r="I54" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>ESTADO_ALEATORIO</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Espinhos tóxicos</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Reflexo</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Tem {rng} de chance de deixar um rival aleatório {T} ao ser atingido.</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>3</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>6</v>
+      </c>
+      <c r="I55" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>ESTADO_DEVOLVE</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Sincronia</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Ao receber um estado</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Tem {rng} de chance de devolver a quem o causou o estado alterado recebido.</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>2</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>20</v>
+      </c>
+      <c r="I56" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>IMUNE_ESTADO</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Imunidade a estado</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Passivo</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Imunidade a estados alterados: {T}.</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>0</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>FORCA_ESTADO</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Força sob estado</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Com estado alterado</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Enquanto estiver com {T}, os golpes causam {rng} mais dano.</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>0</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
+        <v>10</v>
+      </c>
+      <c r="I58" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>DEFESA_ESTADO</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Defesa sob estado</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Com estado alterado</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Enquanto estiver com {T}, recebe {rng} menos dano.</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>0</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>10</v>
+      </c>
+      <c r="I59" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>AGILIDADE_ESTADO</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Agilidade sob estado</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Com estado alterado</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Enquanto estiver com {T}, ganha {rng} de Agilidade.</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>0</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Agilidade</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>10</v>
+      </c>
+      <c r="I60" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>CURA_VENENO</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Cura tóxica</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Envenenado</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Quando envenenado, em vez de perder HP recupera {rng} do HP máximo no fim do turno.</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>0</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="H61" t="n">
+        <v>5</v>
+      </c>
+      <c r="I61" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>DANO_CONTRA_ESTADO</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Aproveitar a fraqueza</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Golpes contra alvos {T} causam {rng} mais dano.</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>3</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="H62" t="n">
+        <v>12</v>
+      </c>
+      <c r="I62" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>BONUS_CHANCE_ESTADO</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Provocar estados</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Passivo</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Soma {rng} (pontos percentuais) à chance dos estados alterados aplicados pelas habilidades dos aliados.</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>0</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="H63" t="n">
+        <v>3</v>
+      </c>
+      <c r="I63" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>IGNORA_IMUNIDADE</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Corrosão</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Controle</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Passivo</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Os estados de veneno dos aliados têm {rng} de chance de ignorar a imunidade de mascotes Veneno e Metal.</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>0</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="H64" t="n">
+        <v>10</v>
+      </c>
+      <c r="I64" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>CLIMA_CHUVA</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Chuva</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Início da luta</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Terreno de chuva: nas 3 primeiras rodadas, aliados do tipo {T} ganham {rng} de Agilidade.</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>3</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="H65" t="n">
+        <v>9</v>
+      </c>
+      <c r="I65" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>CLIMA_AREIA</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Tempestade de areia</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Início da luta</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Nas 3 primeiras rodadas, todos os mascotes que não são dos tipos Pedra, Terra ou Metal perdem 3% do HP máximo no início da rodada.</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>3</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>CLIMA_AREIA_REACAO</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Areia reativa</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Tem {rng} de chance, ao ser atingido, de criar uma tempestade de areia na rodada seguinte (quem não é Pedra, Terra ou Metal perde 3% do HP máximo).</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>3</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="H67" t="n">
+        <v>6</v>
+      </c>
+      <c r="I67" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>CURA_CLIMA</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Pele hidratada</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Ao agir na chuva</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Em terreno de chuva, antes de atacar recupera {rng} do HP máximo.</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>3</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="H68" t="n">
+        <v>5</v>
+      </c>
+      <c r="I68" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>ATRIBUTO_CLIMA</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Impulso do sol</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Sob sol forte</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Sob sol forte, o maior atributo do mascote sobe {rng}: Força e Instinto viram mais dano, Agilidade vira velocidade e Vitalidade vira menos dano recebido.</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>2</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="H69" t="n">
+        <v>8</v>
+      </c>
+      <c r="I69" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>ARMADURA_FRACA</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Armadura quebrada</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Suporte</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Ao ser atingido pela primeira vez, passa a receber 10% mais dano, mas ganha {rng} de Agilidade pelo resto da luta.</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Agilidade</t>
+        </is>
+      </c>
+      <c r="H70" t="n">
+        <v>14</v>
+      </c>
+      <c r="I70" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>COPIA_TIPO_ALIADO</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Disfarce</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Primeira ação</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Na primeira ação, assume o tipo do primeiro mascote do próprio time e ganha {rng} de Vitalidade (menos dano recebido) por 2 rodadas.</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Agilidade</t>
+        </is>
+      </c>
+      <c r="H71" t="n">
+        <v>6</v>
+      </c>
+      <c r="I71" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>COPIA_TIPO_RIVAL</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Impostor</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Primeira ação</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Na primeira ação, assume o tipo do primeiro rival em campo e ganha {rng} de Agilidade por 2 rodadas.</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="H72" t="n">
+        <v>6</v>
+      </c>
+      <c r="I72" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>CONVERSAO_TIPO</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Conversão de tipo</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Se o mascote é do tipo Normal, tem {rng} de chance de o golpe virar {T} e ser super efetivo (+30% de dano) contra mascotes fracos a esse tipo.</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>2</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Força</t>
+        </is>
+      </c>
+      <c r="H73" t="n">
+        <v>20</v>
+      </c>
+      <c r="I73" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ANULA_DEBUFF</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Anular debuff</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Ao receber debuff</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Tem {rng} de chance de ignorar um debuff recebido.</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>3</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="H74" t="n">
+        <v>5</v>
+      </c>
+      <c r="I74" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>ATAQUE_RAPIDO</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Garra rápida</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Primeira rodada</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Na 1ª rodada, ganha {rng} de Agilidade e age primeiro.</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Agilidade</t>
+        </is>
+      </c>
+      <c r="H75" t="n">
+        <v>12</v>
+      </c>
+      <c r="I75" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>IGNORA_PROVOCADOR</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Alvo firme</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Ao atacar</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Tem {rng} de chance de ignorar um Provocador e manter o alvo escolhido.</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>3</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Agilidade</t>
+        </is>
+      </c>
+      <c r="H76" t="n">
+        <v>6</v>
+      </c>
+      <c r="I76" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>ATACA_APESAR_ESTADO</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Mente aberta</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Ao agir com estado</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Tem {rng} de chance de ignorar um estado que o impediria de agir (sono, paralisia ou confusão).</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>2</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="H77" t="n">
+        <v>15</v>
+      </c>
+      <c r="I77" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>COPIA_BUFF</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Copiar buff</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Rival ganha buff</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Tem {rng} de chance de copiar por 2 rodadas um buff que um rival receber (um por vez).</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>2</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="H78" t="n">
+        <v>10</v>
+      </c>
+      <c r="I78" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>MUDANCA_STATUS</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Mudança de status</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Controle</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Início da luta</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Embaralha os atributos do rival mais forte: o maior atributo dele cai {rng}.</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="H79" t="n">
+        <v>6</v>
+      </c>
+      <c r="I79" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>GUARDA_TIPO</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Proteção de tipo</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Ao proteger</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Quando o Guardião protege um aliado do tipo {T}, o golpe causa {rng} menos dano.</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="H80" t="n">
+        <v>9</v>
+      </c>
+      <c r="I80" t="n">
         <v>15</v>
       </c>
     </row>
@@ -2572,7 +3708,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O307"/>
+  <dimension ref="A1:O313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2751,12 +3887,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Maestria elemental</t>
+          <t>Conversão de tipo</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>MAESTRIA_TIPO</t>
+          <t>CONVERSAO_TIPO</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -2771,7 +3907,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Se o mascote tem o tipo Voador, seus golpes causam 6% a 20% mais dano.</t>
+          <t>Se o mascote é do tipo Normal, tem {rng} de chance de o golpe virar {T} e ser super efetivo (+30% de dano) contra mascotes fracos a esse tipo.</t>
         </is>
       </c>
       <c r="I3" t="n">
@@ -2783,10 +3919,10 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L3" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="M3" t="n">
         <v>2</v>
@@ -3433,7 +4569,7 @@
         <v>20</v>
       </c>
       <c r="M13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -3497,7 +4633,7 @@
         <v>20</v>
       </c>
       <c r="M14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -3645,27 +4781,32 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Controle</t>
+          <t>Dano</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Pesadelo</t>
+          <t>Aproveitar a fraqueza</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>PESADELO</t>
+          <t>DANO_CONTRA_ESTADO</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>dormindo</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Início da rodada</t>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, cada rival perde 2% a 6% do HP máximo no início da rodada.</t>
+          <t>Golpes contra alvos {T} causam {rng} mais dano.</t>
         </is>
       </c>
       <c r="I17" t="n">
@@ -3673,14 +4814,14 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Instinto</t>
+          <t>Força</t>
         </is>
       </c>
       <c r="K17" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="L17" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="M17" t="n">
         <v>1</v>
@@ -3692,7 +4833,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>Machuca rivais dormindo a cada turno.</t>
+          <t>Machuca rivais dormindo (dano extra contra alvos dormindo).</t>
         </is>
       </c>
     </row>
@@ -4556,12 +5697,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Resistência a debuff</t>
+          <t>Anular debuff</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>CORPO_LIMPO</t>
+          <t>ANULA_DEBUFF</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -4571,11 +5712,11 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Debuffs recebidos ficam 8% a 20% menores.</t>
+          <t>Tem {rng} de chance de ignorar um debuff recebido.</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -4583,10 +5724,10 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="L31" t="n">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="M31" t="n">
         <v>19</v>
@@ -4742,37 +5883,31 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Resistência a debuff</t>
+          <t>Imunidade a estado</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>CORPO_LIMPO</t>
+          <t>IMUNE_ESTADO</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Todos os estados alterados</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Passivo</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Debuffs recebidos ficam 8% a 20% menores.</t>
+          <t>Imunidade a estados alterados: {T}.</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>3</v>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>Vitalidade</t>
-        </is>
-      </c>
-      <c r="K34" t="n">
-        <v>8</v>
-      </c>
-      <c r="L34" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="M34" t="n">
         <v>1</v>
@@ -5062,31 +6197,26 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Toque debilitante</t>
+          <t>Corrosão</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>TOQUE</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Vitalidade</t>
+          <t>IGNORA_IMUNIDADE</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Ao atacar</t>
+          <t>Passivo</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>30% de chance de reduzir Vitalidade do alvo em 6% a 20%.</t>
+          <t>Os estados de veneno dos aliados têm {rng} de chance de ignorar a imunidade de mascotes Veneno e Metal.</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -5094,7 +6224,7 @@
         </is>
       </c>
       <c r="K39" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L39" t="n">
         <v>20</v>
@@ -5109,7 +6239,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>Pode envenenar Pokémon de Aço e Veneno.</t>
+          <t>Pode envenenar Pokémon de Metal e Veneno (os aliados ignoram a imunidade).</t>
         </is>
       </c>
     </row>
@@ -5328,17 +6458,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Reação de contato</t>
+          <t>Contágio</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>REACAO</t>
+          <t>ESTADO_CONTATO</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Instinto</t>
+          <t>maldito</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -5348,7 +6478,7 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>30% de chance de reduzir Instinto do atacante em 6% a 20%.</t>
+          <t>Tem {rng} de chance de deixar o atacante {T} (um estado por vez).</t>
         </is>
       </c>
       <c r="I43" t="n">
@@ -5360,10 +6490,10 @@
         </is>
       </c>
       <c r="K43" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L43" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="M43" t="n">
         <v>13</v>
@@ -5997,7 +7127,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Fogo</t>
+          <t>Fogo e Planta</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -6007,7 +7137,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Fogo causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo {T} causam {rng} mais dano.</t>
         </is>
       </c>
       <c r="I53" t="n">
@@ -6322,12 +7452,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Ambiente</t>
+          <t>Chuva</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>AMBIENTE</t>
+          <t>CLIMA_CHUVA</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -6342,7 +7472,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Água causam 4% a 12% mais dano.</t>
+          <t>Terreno de chuva: nas 3 primeiras rodadas, aliados do tipo {T} ganham {rng} de Agilidade.</t>
         </is>
       </c>
       <c r="I58" t="n">
@@ -6354,10 +7484,10 @@
         </is>
       </c>
       <c r="K58" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="L58" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="M58" t="n">
         <v>3</v>
@@ -6401,7 +7531,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Fogo</t>
+          <t>Fogo e Planta</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -6411,7 +7541,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Fogo causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo {T} causam {rng} mais dano.</t>
         </is>
       </c>
       <c r="I59" t="n">
@@ -6460,22 +7590,22 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Cura gradual</t>
+          <t>Pele hidratada</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>CURA_GRADUAL</t>
+          <t>CURA_CLIMA</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Início da rodada</t>
+          <t>Ao agir na chuva</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Cura 3% a 10% do HP máximo.</t>
+          <t>Em terreno de chuva, antes de atacar recupera {rng} do HP máximo.</t>
         </is>
       </c>
       <c r="I60" t="n">
@@ -6487,7 +7617,7 @@
         </is>
       </c>
       <c r="K60" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L60" t="n">
         <v>10</v>
@@ -6502,7 +7632,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>Recupera HP na chuva e perde sob sol forte.</t>
+          <t>Recupera HP na chuva.</t>
         </is>
       </c>
     </row>
@@ -6726,17 +7856,17 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Reação de contato</t>
+          <t>Contágio</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>REACAO</t>
+          <t>ESTADO_CONTATO</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Instinto</t>
+          <t>paralisado, envenenado ou dormindo (aleatório)</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -6746,11 +7876,11 @@
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>30% de chance de reduzir Instinto do atacante em 6% a 20%.</t>
+          <t>Tem {rng} de chance de deixar o atacante {T} (um estado por vez).</t>
         </is>
       </c>
       <c r="I64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
@@ -6761,7 +7891,7 @@
         <v>6</v>
       </c>
       <c r="L64" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="M64" t="n">
         <v>11</v>
@@ -6943,7 +8073,7 @@
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>O próximo golpe recebido causa 8% a 20% menos dano.</t>
+          <t>O próximo golpe recebido causa {rng} menos dano.</t>
         </is>
       </c>
       <c r="I67" t="n">
@@ -6955,10 +8085,10 @@
         </is>
       </c>
       <c r="K67" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="L67" t="n">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="M67" t="n">
         <v>1</v>
@@ -6970,7 +8100,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>Sai de campo quando o HP cai abaixo da metade.</t>
+          <t>Sai de campo quando o HP cai abaixo da metade (aqui: reduz o golpe seguinte).</t>
         </is>
       </c>
     </row>
@@ -7194,17 +8324,17 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Reação de contato</t>
+          <t>Contágio</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>REACAO</t>
+          <t>ESTADO_CONTATO</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Força</t>
+          <t>queimado</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -7214,11 +8344,11 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>30% de chance de reduzir Força do atacante em 6% a 20%.</t>
+          <t>Tem {rng} de chance de deixar o atacante {T} (um estado por vez).</t>
         </is>
       </c>
       <c r="I71" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J71" t="inlineStr">
         <is>
@@ -7229,7 +8359,7 @@
         <v>6</v>
       </c>
       <c r="L71" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="M71" t="n">
         <v>23</v>
@@ -7263,26 +8393,31 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Adversidade</t>
+          <t>Força sob estado</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>ADVERSIDADE</t>
+          <t>FORCA_ESTADO</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>o estado queimado</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Com estado alterado</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Ao ter um atributo reduzido, o próximo golpe causa 8% a 20% mais dano.</t>
+          <t>Enquanto estiver com {T}, os golpes causam {rng} mais dano.</t>
         </is>
       </c>
       <c r="I72" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J72" t="inlineStr">
         <is>
@@ -7290,10 +8425,10 @@
         </is>
       </c>
       <c r="K72" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L72" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="M72" t="n">
         <v>2</v>
@@ -8622,26 +9757,31 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Adversidade</t>
+          <t>Força sob estado</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>ADVERSIDADE</t>
+          <t>FORCA_ESTADO</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>qualquer estado alterado</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Com estado alterado</t>
         </is>
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Ao ter um atributo reduzido, o próximo golpe causa 8% a 20% mais dano.</t>
+          <t>Enquanto estiver com {T}, os golpes causam {rng} mais dano.</t>
         </is>
       </c>
       <c r="I93" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J93" t="inlineStr">
         <is>
@@ -8649,10 +9789,10 @@
         </is>
       </c>
       <c r="K93" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L93" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="M93" t="n">
         <v>26</v>
@@ -9720,26 +10860,26 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Evasiva</t>
+          <t>Disfarce</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>EVASIVA</t>
+          <t>COPIA_TIPO_ALIADO</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>Ao ser atingido</t>
+          <t>Primeira ação</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>Esquiva parcial: o golpe causa 4% a 12% menos dano.</t>
+          <t>Na primeira ação, assume o tipo do primeiro mascote do próprio time e ganha {rng} de Vitalidade (menos dano recebido) por 2 rodadas.</t>
         </is>
       </c>
       <c r="I110" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J110" t="inlineStr">
         <is>
@@ -9747,10 +10887,10 @@
         </is>
       </c>
       <c r="K110" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L110" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="M110" t="n">
         <v>2</v>
@@ -9784,37 +10924,31 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Resistência a debuff</t>
+          <t>Imunidade a estado</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>CORPO_LIMPO</t>
+          <t>IMUNE_ESTADO</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Envenenado</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Passivo</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
         <is>
-          <t>Debuffs recebidos ficam 8% a 20% menores.</t>
+          <t>Imunidade a estados alterados: {T}.</t>
         </is>
       </c>
       <c r="I111" t="n">
-        <v>3</v>
-      </c>
-      <c r="J111" t="inlineStr">
-        <is>
-          <t>Vitalidade</t>
-        </is>
-      </c>
-      <c r="K111" t="n">
-        <v>8</v>
-      </c>
-      <c r="L111" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="M111" t="n">
         <v>4</v>
@@ -9848,26 +10982,26 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Espelho</t>
+          <t>Impostor</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>ESPELHO</t>
+          <t>COPIA_TIPO_RIVAL</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Primeira ação</t>
         </is>
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>Devolve 6% a 20% do debuff recebido a quem o aplicou.</t>
+          <t>Na primeira ação, assume o tipo do primeiro rival em campo e ganha {rng} de Agilidade por 2 rodadas.</t>
         </is>
       </c>
       <c r="I112" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J112" t="inlineStr">
         <is>
@@ -9878,7 +11012,7 @@
         <v>6</v>
       </c>
       <c r="L112" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="M112" t="n">
         <v>1</v>
@@ -10104,37 +11238,31 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Resistência a debuff</t>
+          <t>Imunidade a estado</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>CORPO_LIMPO</t>
+          <t>IMUNE_ESTADO</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>Dormindo</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Passivo</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>Debuffs recebidos ficam 8% a 20% menores.</t>
+          <t>Imunidade a estados alterados: {T}.</t>
         </is>
       </c>
       <c r="I116" t="n">
-        <v>3</v>
-      </c>
-      <c r="J116" t="inlineStr">
-        <is>
-          <t>Vitalidade</t>
-        </is>
-      </c>
-      <c r="K116" t="n">
-        <v>8</v>
-      </c>
-      <c r="L116" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="M116" t="n">
         <v>24</v>
@@ -10626,37 +11754,31 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Resistência a debuff</t>
+          <t>Imunidade a estado</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>CORPO_LIMPO</t>
+          <t>IMUNE_ESTADO</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>Todos os estados alterados (sob sol forte)</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Passivo</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>Debuffs recebidos ficam 8% a 20% menores.</t>
+          <t>Imunidade a estados alterados: {T}.</t>
         </is>
       </c>
       <c r="I124" t="n">
-        <v>3</v>
-      </c>
-      <c r="J124" t="inlineStr">
-        <is>
-          <t>Vitalidade</t>
-        </is>
-      </c>
-      <c r="K124" t="n">
-        <v>8</v>
-      </c>
-      <c r="L124" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="M124" t="n">
         <v>22</v>
@@ -10690,12 +11812,12 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Absorção</t>
+          <t>Pelagem elemental</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>ABSORCAO</t>
+          <t>PELAGEM</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -10710,7 +11832,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>Golpes do tipo Terra causam 6% a 20% menos dano e curam 5% do HP máximo.</t>
+          <t>Golpes {T} causam {rng} menos dano.</t>
         </is>
       </c>
       <c r="I125" t="n">
@@ -10722,10 +11844,10 @@
         </is>
       </c>
       <c r="K125" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L125" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="M125" t="n">
         <v>65</v>
@@ -10956,37 +12078,31 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Resistência a debuff</t>
+          <t>Imunidade a estado</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>CORPO_LIMPO</t>
+          <t>IMUNE_ESTADO</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Paralisado</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Passivo</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
         <is>
-          <t>Debuffs recebidos ficam 8% a 20% menores.</t>
+          <t>Imunidade a estados alterados: {T}.</t>
         </is>
       </c>
       <c r="I129" t="n">
-        <v>3</v>
-      </c>
-      <c r="J129" t="inlineStr">
-        <is>
-          <t>Vitalidade</t>
-        </is>
-      </c>
-      <c r="K129" t="n">
-        <v>8</v>
-      </c>
-      <c r="L129" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="M129" t="n">
         <v>14</v>
@@ -11153,12 +12269,12 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Maestria elemental</t>
+          <t>Conversão de tipo</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>MAESTRIA_TIPO</t>
+          <t>CONVERSAO_TIPO</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -11173,7 +12289,7 @@
       </c>
       <c r="H132" t="inlineStr">
         <is>
-          <t>Se o mascote tem o tipo Água, seus golpes causam 6% a 20% mais dano.</t>
+          <t>Se o mascote é do tipo Normal, tem {rng} de chance de o golpe virar {T} e ser super efetivo (+30% de dano) contra mascotes fracos a esse tipo.</t>
         </is>
       </c>
       <c r="I132" t="n">
@@ -11185,10 +12301,10 @@
         </is>
       </c>
       <c r="K132" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L132" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="M132" t="n">
         <v>3</v>
@@ -11472,37 +12588,31 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Resistência a debuff</t>
+          <t>Imunidade a estado</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>CORPO_LIMPO</t>
+          <t>IMUNE_ESTADO</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Congelado</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Passivo</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
         <is>
-          <t>Debuffs recebidos ficam 8% a 20% menores.</t>
+          <t>Imunidade a estados alterados: {T}.</t>
         </is>
       </c>
       <c r="I137" t="n">
-        <v>3</v>
-      </c>
-      <c r="J137" t="inlineStr">
-        <is>
-          <t>Vitalidade</t>
-        </is>
-      </c>
-      <c r="K137" t="n">
-        <v>8</v>
-      </c>
-      <c r="L137" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="M137" t="n">
         <v>3</v>
@@ -11583,7 +12693,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>Impede rivais de Aço de fugir ou trocar.</t>
+          <t>Impede rivais de Metal de fugir ou trocar.</t>
         </is>
       </c>
     </row>
@@ -11605,26 +12715,31 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Postura firme</t>
+          <t>Defesa sob estado</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>PREPARO</t>
+          <t>DEFESA_ESTADO</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>qualquer estado alterado</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
         <is>
-          <t>Ao preparar defesa</t>
+          <t>Com estado alterado</t>
         </is>
       </c>
       <c r="H139" t="inlineStr">
         <is>
-          <t>Ao preparar defesa (Defensor), reduz 6% a 20% extra do próximo golpe.</t>
+          <t>Enquanto estiver com {T}, recebe {rng} menos dano.</t>
         </is>
       </c>
       <c r="I139" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J139" t="inlineStr">
         <is>
@@ -11632,10 +12747,10 @@
         </is>
       </c>
       <c r="K139" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L139" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="M139" t="n">
         <v>3</v>
@@ -11748,7 +12863,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>Fogo</t>
+          <t>Fogo e Planta</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -11758,7 +12873,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Fogo causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo {T} causam {rng} mais dano.</t>
         </is>
       </c>
       <c r="I141" t="n">
@@ -11807,12 +12922,17 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Golpe certeiro</t>
+          <t>Aproveitar a fraqueza</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>QUEBRA_GUARDA</t>
+          <t>DANO_CONTRA_ESTADO</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>envenenados</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -11822,19 +12942,19 @@
       </c>
       <c r="H142" t="inlineStr">
         <is>
-          <t>Ignora 6% a 20% da mitigação (Vitalidade) do alvo.</t>
+          <t>Golpes contra alvos {T} causam {rng} mais dano.</t>
         </is>
       </c>
       <c r="I142" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J142" t="inlineStr">
         <is>
-          <t>Instinto</t>
+          <t>Força</t>
         </is>
       </c>
       <c r="K142" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L142" t="n">
         <v>20</v>
@@ -12904,22 +14024,22 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Golpe certeiro</t>
+          <t>Mente aberta</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>QUEBRA_GUARDA</t>
+          <t>ATACA_APESAR_ESTADO</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>Ao atacar</t>
+          <t>Ao agir com estado</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Ignora 6% a 20% da mitigação (Vitalidade) do alvo.</t>
+          <t>Tem {rng} de chance de ignorar um estado que o impediria de agir (sono, paralisia ou confusão).</t>
         </is>
       </c>
       <c r="I159" t="n">
@@ -12931,10 +14051,10 @@
         </is>
       </c>
       <c r="K159" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="L159" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="M159" t="n">
         <v>13</v>
@@ -13175,7 +14295,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>Fogo</t>
+          <t>Fogo e Planta</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -13185,7 +14305,7 @@
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Fogo causam 4% a 12% mais dano.</t>
+          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo {T} causam {rng} mais dano.</t>
         </is>
       </c>
       <c r="I163" t="n">
@@ -13367,37 +14487,31 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Resistência a debuff</t>
+          <t>Imunidade a estado</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>CORPO_LIMPO</t>
+          <t>IMUNE_ESTADO</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>Confuso</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Passivo</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Debuffs recebidos ficam 8% a 20% menores.</t>
+          <t>Imunidade a estados alterados: {T}.</t>
         </is>
       </c>
       <c r="I166" t="n">
-        <v>3</v>
-      </c>
-      <c r="J166" t="inlineStr">
-        <is>
-          <t>Vitalidade</t>
-        </is>
-      </c>
-      <c r="K166" t="n">
-        <v>8</v>
-      </c>
-      <c r="L166" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="M166" t="n">
         <v>30</v>
@@ -13495,26 +14609,26 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Espinhos</t>
+          <t>Último suspiro</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>ESPINHOS</t>
+          <t>ULTIMO_SUSPIRO</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>Ao ser atingido</t>
+          <t>Ao ser derrotado</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Devolve 6% a 20% do dano recebido ao atacante (mínimo 1).</t>
+          <t>Ao cair, causa {rng} do HP máximo dele ao último atacante.</t>
         </is>
       </c>
       <c r="I168" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J168" t="inlineStr">
         <is>
@@ -13522,10 +14636,10 @@
         </is>
       </c>
       <c r="K168" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="L168" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="M168" t="n">
         <v>1</v>
@@ -13751,12 +14865,12 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Maestria elemental</t>
+          <t>Conversão de tipo</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>MAESTRIA_TIPO</t>
+          <t>CONVERSAO_TIPO</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -13771,7 +14885,7 @@
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>Se o mascote tem o tipo Fada, seus golpes causam 6% a 20% mais dano.</t>
+          <t>Se o mascote é do tipo Normal, tem {rng} de chance de o golpe virar {T} e ser super efetivo (+30% de dano) contra mascotes fracos a esse tipo.</t>
         </is>
       </c>
       <c r="I172" t="n">
@@ -13783,10 +14897,10 @@
         </is>
       </c>
       <c r="K172" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L172" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="M172" t="n">
         <v>3</v>
@@ -13884,26 +14998,26 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Cura gradual</t>
+          <t>Cura tóxica</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>CURA_GRADUAL</t>
+          <t>CURA_VENENO</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
         <is>
-          <t>Início da rodada</t>
+          <t>Envenenado</t>
         </is>
       </c>
       <c r="H174" t="inlineStr">
         <is>
-          <t>Cura 3% a 10% do HP máximo.</t>
+          <t>Quando envenenado, em vez de perder HP recupera {rng} do HP máximo no fim do turno.</t>
         </is>
       </c>
       <c r="I174" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J174" t="inlineStr">
         <is>
@@ -13911,7 +15025,7 @@
         </is>
       </c>
       <c r="K174" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="L174" t="n">
         <v>10</v>
@@ -13948,17 +15062,17 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Reação de contato</t>
+          <t>Contágio</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>REACAO</t>
+          <t>ESTADO_CONTATO</t>
         </is>
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t>Vitalidade</t>
+          <t>envenenado</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -13968,11 +15082,11 @@
       </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>30% de chance de reduzir Vitalidade do atacante em 6% a 20%.</t>
+          <t>Tem {rng} de chance de deixar o atacante {T} (um estado por vez).</t>
         </is>
       </c>
       <c r="I175" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J175" t="inlineStr">
         <is>
@@ -13983,7 +15097,7 @@
         <v>6</v>
       </c>
       <c r="L175" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="M175" t="n">
         <v>19</v>
@@ -14017,17 +15131,17 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Toque debilitante</t>
+          <t>Toque de estado</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>TOQUE</t>
+          <t>ESTADO_TOQUE</t>
         </is>
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>Instinto</t>
+          <t>confuso</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
@@ -14037,7 +15151,7 @@
       </c>
       <c r="H176" t="inlineStr">
         <is>
-          <t>30% de chance de reduzir Instinto do alvo em 6% a 20%.</t>
+          <t>Tem {rng} de chance de deixar o alvo {T} ao atacar (um estado por vez).</t>
         </is>
       </c>
       <c r="I176" t="n">
@@ -14052,7 +15166,7 @@
         <v>6</v>
       </c>
       <c r="L176" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="M176" t="n">
         <v>1</v>
@@ -14086,17 +15200,17 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Toque debilitante</t>
+          <t>Toque de estado</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>TOQUE</t>
+          <t>ESTADO_TOQUE</t>
         </is>
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>Vitalidade</t>
+          <t>envenenado</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
@@ -14106,11 +15220,11 @@
       </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>30% de chance de reduzir Vitalidade do alvo em 6% a 20%.</t>
+          <t>Tem {rng} de chance de deixar o alvo {T} ao atacar (um estado por vez).</t>
         </is>
       </c>
       <c r="I177" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J177" t="inlineStr">
         <is>
@@ -14121,7 +15235,7 @@
         <v>6</v>
       </c>
       <c r="L177" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="M177" t="n">
         <v>9</v>
@@ -14283,37 +15397,37 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Impulso</t>
+          <t>Provocar estados</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>IMPULSO</t>
+          <t>BONUS_CHANCE_ESTADO</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>Início da rodada</t>
+          <t>Passivo</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, ganha Agilidade, até 4% a 12% no total.</t>
+          <t>Soma {rng} (pontos percentuais) à chance dos estados alterados aplicados pelas habilidades dos aliados.</t>
         </is>
       </c>
       <c r="I180" t="n">
+        <v>0</v>
+      </c>
+      <c r="J180" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K180" t="n">
         <v>3</v>
       </c>
-      <c r="J180" t="inlineStr">
-        <is>
-          <t>Agilidade</t>
-        </is>
-      </c>
-      <c r="K180" t="n">
-        <v>4</v>
-      </c>
       <c r="L180" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="M180" t="n">
         <v>20</v>
@@ -14549,22 +15663,22 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Evasiva</t>
+          <t>Alvo firme</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>EVASIVA</t>
+          <t>IGNORA_PROVOCADOR</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>Ao ser atingido</t>
+          <t>Ao atacar</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>Esquiva parcial: o golpe causa 4% a 12% menos dano.</t>
+          <t>Tem {rng} de chance de ignorar um Provocador e manter o alvo escolhido.</t>
         </is>
       </c>
       <c r="I184" t="n">
@@ -14576,10 +15690,10 @@
         </is>
       </c>
       <c r="K184" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L184" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="M184" t="n">
         <v>2</v>
@@ -14677,22 +15791,22 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Ataque reforçado</t>
+          <t>Impulso do sol</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>PODER_BRUTO</t>
+          <t>ATRIBUTO_CLIMA</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>Ao atacar</t>
+          <t>Sob sol forte</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>Nas duas primeiras ações, o golpe causa 8% a 20% mais dano.</t>
+          <t>Sob sol forte, o maior atributo do mascote sobe {rng}: Força e Instinto viram mais dano, Agilidade vira velocidade e Vitalidade vira menos dano recebido.</t>
         </is>
       </c>
       <c r="I186" t="n">
@@ -14943,37 +16057,31 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Resistência a debuff</t>
+          <t>Imunidade a estado</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>CORPO_LIMPO</t>
+          <t>IMUNE_ESTADO</t>
+        </is>
+      </c>
+      <c r="F190" t="inlineStr">
+        <is>
+          <t>Todos os estados alterados</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Passivo</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>Debuffs recebidos ficam 8% a 20% menores.</t>
+          <t>Imunidade a estados alterados: {T}.</t>
         </is>
       </c>
       <c r="I190" t="n">
-        <v>3</v>
-      </c>
-      <c r="J190" t="inlineStr">
-        <is>
-          <t>Vitalidade</t>
-        </is>
-      </c>
-      <c r="K190" t="n">
-        <v>8</v>
-      </c>
-      <c r="L190" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="M190" t="n">
         <v>3</v>
@@ -15135,42 +16243,47 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Dano</t>
+          <t>Suporte</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Adversidade</t>
+          <t>Agilidade sob estado</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>ADVERSIDADE</t>
+          <t>AGILIDADE_ESTADO</t>
+        </is>
+      </c>
+      <c r="F193" t="inlineStr">
+        <is>
+          <t>qualquer estado alterado</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Com estado alterado</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>Ao ter um atributo reduzido, o próximo golpe causa 8% a 20% mais dano.</t>
+          <t>Enquanto estiver com {T}, ganha {rng} de Agilidade.</t>
         </is>
       </c>
       <c r="I193" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J193" t="inlineStr">
         <is>
-          <t>Força</t>
+          <t>Agilidade</t>
         </is>
       </c>
       <c r="K193" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L193" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="M193" t="n">
         <v>9</v>
@@ -15465,12 +16578,12 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Maestria elemental</t>
+          <t>Conversão de tipo</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>MAESTRIA_TIPO</t>
+          <t>CONVERSAO_TIPO</t>
         </is>
       </c>
       <c r="F198" t="inlineStr">
@@ -15485,7 +16598,7 @@
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>Se o mascote tem o tipo Gelo, seus golpes causam 6% a 20% mais dano.</t>
+          <t>Se o mascote é do tipo Normal, tem {rng} de chance de o golpe virar {T} e ser super efetivo (+30% de dano) contra mascotes fracos a esse tipo.</t>
         </is>
       </c>
       <c r="I198" t="n">
@@ -15497,10 +16610,10 @@
         </is>
       </c>
       <c r="K198" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L198" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="M198" t="n">
         <v>3</v>
@@ -16098,7 +17211,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>Golpes de Pedra, Terra e Aço ficam mais fortes na tempestade de areia.</t>
+          <t>Golpes de Pedra, Terra e Metal ficam mais fortes na tempestade de areia.</t>
         </is>
       </c>
     </row>
@@ -16184,27 +17297,22 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>Ambiente</t>
+          <t>Areia reativa</t>
         </is>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>AMBIENTE</t>
-        </is>
-      </c>
-      <c r="F209" t="inlineStr">
-        <is>
-          <t>Pedra</t>
+          <t>CLIMA_AREIA_REACAO</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>Início da luta</t>
+          <t>Ao ser atingido</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Pedra causam 4% a 12% mais dano.</t>
+          <t>Tem {rng} de chance, ao ser atingido, de criar uma tempestade de areia na rodada seguinte (quem não é Pedra, Terra ou Metal perde 3% do HP máximo).</t>
         </is>
       </c>
       <c r="I209" t="n">
@@ -16216,10 +17324,10 @@
         </is>
       </c>
       <c r="K209" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L209" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="M209" t="n">
         <v>3</v>
@@ -16253,17 +17361,12 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>Ambiente</t>
+          <t>Tempestade de areia</t>
         </is>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>AMBIENTE</t>
-        </is>
-      </c>
-      <c r="F210" t="inlineStr">
-        <is>
-          <t>Pedra</t>
+          <t>CLIMA_AREIA</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
@@ -16273,23 +17376,12 @@
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>Clima ou terreno criado pela habilidade: nas 3 primeiras rodadas, aliados do tipo Pedra causam 4% a 12% mais dano.</t>
+          <t>Nas 3 primeiras rodadas, todos os mascotes que não são dos tipos Pedra, Terra ou Metal perdem 3% do HP máximo no início da rodada.</t>
         </is>
       </c>
       <c r="I210" t="n">
         <v>3</v>
       </c>
-      <c r="J210" t="inlineStr">
-        <is>
-          <t>Instinto</t>
-        </is>
-      </c>
-      <c r="K210" t="n">
-        <v>4</v>
-      </c>
-      <c r="L210" t="n">
-        <v>12</v>
-      </c>
       <c r="M210" t="n">
         <v>5</v>
       </c>
@@ -17444,7 +18536,7 @@
       </c>
       <c r="H228" t="inlineStr">
         <is>
-          <t>Nas 2 primeiras rodadas, recebe 6% a 20% menos dano. A partir da 3ª rodada, os 3 golpes seguintes que ele dá causam 6% a 20% mais dano. Nunca recebe mais dano por causa disto.</t>
+          <t>Nas 2 primeiras rodadas recebe de 10% a 15% menos dano (cresce com a Vitalidade). A partir da 3ª rodada, os 3 golpes seguintes que ele dá causam {rng} mais dano. Nunca recebe mais dano por causa disto.</t>
         </is>
       </c>
       <c r="I228" t="n">
@@ -17456,7 +18548,7 @@
         </is>
       </c>
       <c r="K228" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L228" t="n">
         <v>20</v>
@@ -18069,17 +19161,22 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Reflexo</t>
+          <t>Controle</t>
         </is>
       </c>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Espinhos</t>
+          <t>Contágio</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>ESPINHOS</t>
+          <t>ESTADO_CONTATO</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>queimado</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
@@ -18089,7 +19186,7 @@
       </c>
       <c r="H238" t="inlineStr">
         <is>
-          <t>Devolve 6% a 20% do dano recebido ao atacante (mínimo 1).</t>
+          <t>Tem {rng} de chance de deixar o atacante {T} (um estado por vez).</t>
         </is>
       </c>
       <c r="I238" t="n">
@@ -18097,14 +19194,14 @@
       </c>
       <c r="J238" t="inlineStr">
         <is>
-          <t>Vitalidade</t>
+          <t>Instinto</t>
         </is>
       </c>
       <c r="K238" t="n">
         <v>6</v>
       </c>
       <c r="L238" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="M238" t="n">
         <v>1</v>
@@ -18261,17 +19358,17 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Dano</t>
+          <t>Defesa</t>
         </is>
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Golpe certeiro</t>
+          <t>Alvo firme</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>QUEBRA_GUARDA</t>
+          <t>IGNORA_PROVOCADOR</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
@@ -18281,22 +19378,22 @@
       </c>
       <c r="H241" t="inlineStr">
         <is>
-          <t>Ignora 6% a 20% da mitigação (Vitalidade) do alvo.</t>
+          <t>Tem {rng} de chance de ignorar um Provocador e manter o alvo escolhido.</t>
         </is>
       </c>
       <c r="I241" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>Instinto</t>
+          <t>Agilidade</t>
         </is>
       </c>
       <c r="K241" t="n">
         <v>6</v>
       </c>
       <c r="L241" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="M241" t="n">
         <v>4</v>
@@ -18458,17 +19555,17 @@
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Reação de contato</t>
+          <t>Contágio</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>REACAO</t>
+          <t>ESTADO_CONTATO</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>Agilidade</t>
+          <t>paralisado</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
@@ -18478,11 +19575,11 @@
       </c>
       <c r="H244" t="inlineStr">
         <is>
-          <t>30% de chance de reduzir Agilidade do atacante em 6% a 20%.</t>
+          <t>Tem {rng} de chance de deixar o atacante {T} (um estado por vez).</t>
         </is>
       </c>
       <c r="I244" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J244" t="inlineStr">
         <is>
@@ -18665,7 +19762,7 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>Aço</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
@@ -18675,7 +19772,7 @@
       </c>
       <c r="H247" t="inlineStr">
         <is>
-          <t>Se o mascote tem o tipo Aço, seus golpes causam 6% a 20% mais dano.</t>
+          <t>Se o mascote tem o tipo Metal, seus golpes causam 6% a 20% mais dano.</t>
         </is>
       </c>
       <c r="I247" t="n">
@@ -18702,7 +19799,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>Golpes de Aço ficam mais fortes.</t>
+          <t>Golpes de Metal ficam mais fortes.</t>
         </is>
       </c>
     </row>
@@ -18734,7 +19831,7 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>Aço</t>
+          <t>Metal</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
@@ -18744,7 +19841,7 @@
       </c>
       <c r="H248" t="inlineStr">
         <is>
-          <t>Aura da habilidade: enquanto o mascote estiver em campo, aliados do tipo Aço causam 4% a 12% mais dano nos golpes (2 vezes por luta).</t>
+          <t>Aura da habilidade: enquanto o mascote estiver em campo, aliados do tipo Metal causam 4% a 12% mais dano nos golpes (2 vezes por luta).</t>
         </is>
       </c>
       <c r="I248" t="n">
@@ -18771,7 +19868,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>Golpes de Aço dos aliados ficam mais fortes.</t>
+          <t>Golpes de Metal dos aliados ficam mais fortes.</t>
         </is>
       </c>
     </row>
@@ -19447,42 +20544,36 @@
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Suporte</t>
+          <t>Defesa</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>Véu</t>
+          <t>Imunidade a estado</t>
         </is>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>VEU</t>
+          <t>IMUNE_ESTADO</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>Dormindo (também aliados)</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Passivo</t>
         </is>
       </c>
       <c r="H259" t="inlineStr">
         <is>
-          <t>Debuffs recebidos pelos aliados ficam 6% a 20% menores.</t>
+          <t>Imunidade a estados alterados: {T}.</t>
         </is>
       </c>
       <c r="I259" t="n">
-        <v>2</v>
-      </c>
-      <c r="J259" t="inlineStr">
-        <is>
-          <t>Carisma</t>
-        </is>
-      </c>
-      <c r="K259" t="n">
-        <v>6</v>
-      </c>
-      <c r="L259" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="M259" t="n">
         <v>11</v>
@@ -19713,22 +20804,22 @@
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>Espelho</t>
+          <t>Sincronia</t>
         </is>
       </c>
       <c r="E263" t="inlineStr">
         <is>
-          <t>ESPELHO</t>
+          <t>ESTADO_DEVOLVE</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Ao receber um estado</t>
         </is>
       </c>
       <c r="H263" t="inlineStr">
         <is>
-          <t>Devolve 6% a 20% do debuff recebido a quem o aplicou.</t>
+          <t>Tem {rng} de chance de devolver a quem o causou o estado alterado recebido.</t>
         </is>
       </c>
       <c r="I263" t="n">
@@ -19740,10 +20831,10 @@
         </is>
       </c>
       <c r="K263" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="L263" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="M263" t="n">
         <v>18</v>
@@ -20628,26 +21719,31 @@
       </c>
       <c r="D277" t="inlineStr">
         <is>
-          <t>Adversidade</t>
+          <t>Força sob estado</t>
         </is>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>ADVERSIDADE</t>
+          <t>FORCA_ESTADO</t>
+        </is>
+      </c>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>o estado envenenado</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Com estado alterado</t>
         </is>
       </c>
       <c r="H277" t="inlineStr">
         <is>
-          <t>Ao ter um atributo reduzido, o próximo golpe causa 8% a 20% mais dano.</t>
+          <t>Enquanto estiver com {T}, os golpes causam {rng} mais dano.</t>
         </is>
       </c>
       <c r="I277" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J277" t="inlineStr">
         <is>
@@ -20655,10 +21751,10 @@
         </is>
       </c>
       <c r="K277" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L277" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="M277" t="n">
         <v>1</v>
@@ -20692,17 +21788,17 @@
       </c>
       <c r="D278" t="inlineStr">
         <is>
-          <t>Toque debilitante</t>
+          <t>Toque de estado</t>
         </is>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>TOQUE</t>
+          <t>ESTADO_TOQUE</t>
         </is>
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>Vitalidade</t>
+          <t>envenenado</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
@@ -20712,7 +21808,7 @@
       </c>
       <c r="H278" t="inlineStr">
         <is>
-          <t>30% de chance de reduzir Vitalidade do alvo em 6% a 20%.</t>
+          <t>Tem {rng} de chance de deixar o alvo {T} ao atacar (um estado por vez).</t>
         </is>
       </c>
       <c r="I278" t="n">
@@ -20727,7 +21823,7 @@
         <v>6</v>
       </c>
       <c r="L278" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="M278" t="n">
         <v>3</v>
@@ -20761,12 +21857,17 @@
       </c>
       <c r="D279" t="inlineStr">
         <is>
-          <t>Espinhos</t>
+          <t>Espinhos tóxicos</t>
         </is>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>ESPINHOS</t>
+          <t>ESTADO_ALEATORIO</t>
+        </is>
+      </c>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>envenenado</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
@@ -20776,7 +21877,7 @@
       </c>
       <c r="H279" t="inlineStr">
         <is>
-          <t>Devolve 6% a 20% do dano recebido ao atacante (mínimo 1).</t>
+          <t>Tem {rng} de chance de deixar um rival aleatório {T} ao ser atingido.</t>
         </is>
       </c>
       <c r="I279" t="n">
@@ -20825,22 +21926,22 @@
       </c>
       <c r="D280" t="inlineStr">
         <is>
-          <t>Espelho</t>
+          <t>Copiar buff</t>
         </is>
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>ESPELHO</t>
+          <t>COPIA_BUFF</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Rival ganha buff</t>
         </is>
       </c>
       <c r="H280" t="inlineStr">
         <is>
-          <t>Devolve 6% a 20% do debuff recebido a quem o aplicou.</t>
+          <t>Tem {rng} de chance de copiar por 2 rodadas um buff que um rival receber (um por vez).</t>
         </is>
       </c>
       <c r="I280" t="n">
@@ -20852,10 +21953,10 @@
         </is>
       </c>
       <c r="K280" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="L280" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="M280" t="n">
         <v>8</v>
@@ -21544,37 +22645,31 @@
       </c>
       <c r="D291" t="inlineStr">
         <is>
-          <t>Resistência a debuff</t>
+          <t>Imunidade a estado</t>
         </is>
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>CORPO_LIMPO</t>
+          <t>IMUNE_ESTADO</t>
+        </is>
+      </c>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>Dormindo</t>
         </is>
       </c>
       <c r="G291" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Passivo</t>
         </is>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>Debuffs recebidos ficam 8% a 20% menores.</t>
+          <t>Imunidade a estados alterados: {T}.</t>
         </is>
       </c>
       <c r="I291" t="n">
-        <v>3</v>
-      </c>
-      <c r="J291" t="inlineStr">
-        <is>
-          <t>Vitalidade</t>
-        </is>
-      </c>
-      <c r="K291" t="n">
-        <v>8</v>
-      </c>
-      <c r="L291" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="M291" t="n">
         <v>15</v>
@@ -21948,37 +23043,31 @@
       </c>
       <c r="D297" t="inlineStr">
         <is>
-          <t>Resistência a debuff</t>
+          <t>Imunidade a estado</t>
         </is>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>CORPO_LIMPO</t>
+          <t>IMUNE_ESTADO</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Queimado</t>
         </is>
       </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>Ao receber debuff</t>
+          <t>Passivo</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>Debuffs recebidos ficam 8% a 20% menores.</t>
+          <t>Imunidade a estados alterados: {T}.</t>
         </is>
       </c>
       <c r="I297" t="n">
-        <v>3</v>
-      </c>
-      <c r="J297" t="inlineStr">
-        <is>
-          <t>Vitalidade</t>
-        </is>
-      </c>
-      <c r="K297" t="n">
-        <v>8</v>
-      </c>
-      <c r="L297" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="M297" t="n">
         <v>13</v>
@@ -22012,26 +23101,26 @@
       </c>
       <c r="D298" t="inlineStr">
         <is>
-          <t>Impulso</t>
+          <t>Armadura quebrada</t>
         </is>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>IMPULSO</t>
+          <t>ARMADURA_FRACA</t>
         </is>
       </c>
       <c r="G298" t="inlineStr">
         <is>
-          <t>Início da rodada</t>
+          <t>Ao ser atingido</t>
         </is>
       </c>
       <c r="H298" t="inlineStr">
         <is>
-          <t>Nas 3 primeiras rodadas, ganha Agilidade, até 4% a 12% no total.</t>
+          <t>Ao ser atingido pela primeira vez, passa a receber 10% mais dano, mas ganha {rng} de Agilidade pelo resto da luta.</t>
         </is>
       </c>
       <c r="I298" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J298" t="inlineStr">
         <is>
@@ -22039,10 +23128,10 @@
         </is>
       </c>
       <c r="K298" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="L298" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="M298" t="n">
         <v>24</v>
@@ -22470,22 +23559,22 @@
       </c>
       <c r="D305" t="inlineStr">
         <is>
-          <t>Evasiva</t>
+          <t>Anular debuff</t>
         </is>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>EVASIVA</t>
+          <t>ANULA_DEBUFF</t>
         </is>
       </c>
       <c r="G305" t="inlineStr">
         <is>
-          <t>Ao ser atingido</t>
+          <t>Ao receber debuff</t>
         </is>
       </c>
       <c r="H305" t="inlineStr">
         <is>
-          <t>Esquiva parcial: o golpe causa 4% a 12% menos dano.</t>
+          <t>Tem {rng} de chance de ignorar um debuff recebido.</t>
         </is>
       </c>
       <c r="I305" t="n">
@@ -22493,14 +23582,14 @@
       </c>
       <c r="J305" t="inlineStr">
         <is>
-          <t>Agilidade</t>
+          <t>Vitalidade</t>
         </is>
       </c>
       <c r="K305" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L305" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="M305" t="n">
         <v>5</v>
@@ -22641,6 +23730,405 @@
       <c r="O307" t="inlineStr">
         <is>
           <t>Assume a forma Heroica ao sair de campo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Transform</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>transform</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>Impostor</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>COPIA_TIPO_RIVAL</t>
+        </is>
+      </c>
+      <c r="G308" t="inlineStr">
+        <is>
+          <t>Primeira ação</t>
+        </is>
+      </c>
+      <c r="H308" t="inlineStr">
+        <is>
+          <t>Na primeira ação, assume o tipo do primeiro rival em campo e ganha {rng} de Agilidade por 2 rodadas.</t>
+        </is>
+      </c>
+      <c r="I308" t="n">
+        <v>1</v>
+      </c>
+      <c r="J308" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K308" t="n">
+        <v>6</v>
+      </c>
+      <c r="L308" t="n">
+        <v>10</v>
+      </c>
+      <c r="M308" t="n">
+        <v>2</v>
+      </c>
+      <c r="N308" t="inlineStr">
+        <is>
+          <t>Transform</t>
+        </is>
+      </c>
+      <c r="O308" t="inlineStr">
+        <is>
+          <t>Transforma-se no rival ao entrar (aqui: copia o tipo dele). Exclusiva de Mew e Ditto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Wonder Room</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>wonder-room</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Controle</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>Mudança de status</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>MUDANCA_STATUS</t>
+        </is>
+      </c>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>Psíquico</t>
+        </is>
+      </c>
+      <c r="G309" t="inlineStr">
+        <is>
+          <t>Início da luta</t>
+        </is>
+      </c>
+      <c r="H309" t="inlineStr">
+        <is>
+          <t>Embaralha os atributos do rival mais forte: o maior atributo dele cai {rng}.</t>
+        </is>
+      </c>
+      <c r="I309" t="n">
+        <v>1</v>
+      </c>
+      <c r="J309" t="inlineStr">
+        <is>
+          <t>Instinto</t>
+        </is>
+      </c>
+      <c r="K309" t="n">
+        <v>6</v>
+      </c>
+      <c r="L309" t="n">
+        <v>12</v>
+      </c>
+      <c r="M309" t="n">
+        <v>6</v>
+      </c>
+      <c r="N309" t="inlineStr">
+        <is>
+          <t>Wonder Room</t>
+        </is>
+      </c>
+      <c r="O309" t="inlineStr">
+        <is>
+          <t>Embaralha os atributos em campo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Endeavor</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>endeavor</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>Vingança</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>VINGANCA</t>
+        </is>
+      </c>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="G310" t="inlineStr">
+        <is>
+          <t>Aliado cai</t>
+        </is>
+      </c>
+      <c r="H310" t="inlineStr">
+        <is>
+          <t>Quando um aliado cai, o próximo golpe causa {rng} mais dano.</t>
+        </is>
+      </c>
+      <c r="I310" t="n">
+        <v>2</v>
+      </c>
+      <c r="J310" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K310" t="n">
+        <v>3</v>
+      </c>
+      <c r="L310" t="n">
+        <v>9</v>
+      </c>
+      <c r="M310" t="n">
+        <v>7</v>
+      </c>
+      <c r="N310" t="inlineStr">
+        <is>
+          <t>Endeavor</t>
+        </is>
+      </c>
+      <c r="O310" t="inlineStr">
+        <is>
+          <t>Revida quando o time está em desvantagem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Air Balloon</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>air-balloon</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Evasiva</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>EVASIVA</t>
+        </is>
+      </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>Ao ser atingido</t>
+        </is>
+      </c>
+      <c r="H311" t="inlineStr">
+        <is>
+          <t>Esquiva parcial: o golpe causa {rng} menos dano.</t>
+        </is>
+      </c>
+      <c r="I311" t="n">
+        <v>1</v>
+      </c>
+      <c r="J311" t="inlineStr">
+        <is>
+          <t>Carisma</t>
+        </is>
+      </c>
+      <c r="K311" t="n">
+        <v>12</v>
+      </c>
+      <c r="L311" t="n">
+        <v>20</v>
+      </c>
+      <c r="M311" t="n">
+        <v>8</v>
+      </c>
+      <c r="N311" t="inlineStr">
+        <is>
+          <t>Air Balloon</t>
+        </is>
+      </c>
+      <c r="O311" t="inlineStr">
+        <is>
+          <t>Flutua com um balão: esquiva parcial.</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Lum Protection</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>lum-protection</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Defesa</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Proteção de tipo</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>GUARDA_TIPO</t>
+        </is>
+      </c>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>Voador</t>
+        </is>
+      </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>Ao proteger</t>
+        </is>
+      </c>
+      <c r="H312" t="inlineStr">
+        <is>
+          <t>Quando o Guardião protege um aliado do tipo {T}, o golpe causa {rng} menos dano.</t>
+        </is>
+      </c>
+      <c r="I312" t="n">
+        <v>1</v>
+      </c>
+      <c r="J312" t="inlineStr">
+        <is>
+          <t>Vitalidade</t>
+        </is>
+      </c>
+      <c r="K312" t="n">
+        <v>9</v>
+      </c>
+      <c r="L312" t="n">
+        <v>15</v>
+      </c>
+      <c r="M312" t="n">
+        <v>9</v>
+      </c>
+      <c r="N312" t="inlineStr">
+        <is>
+          <t>Lum Protection</t>
+        </is>
+      </c>
+      <c r="O312" t="inlineStr">
+        <is>
+          <t>Protege aliados com a força das aves.</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Quick Claw</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>quick-claw</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Dano</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Garra rápida</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>ATAQUE_RAPIDO</t>
+        </is>
+      </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>Primeira rodada</t>
+        </is>
+      </c>
+      <c r="H313" t="inlineStr">
+        <is>
+          <t>Na 1ª rodada, ganha {rng} de Agilidade e age primeiro.</t>
+        </is>
+      </c>
+      <c r="I313" t="n">
+        <v>1</v>
+      </c>
+      <c r="J313" t="inlineStr">
+        <is>
+          <t>Agilidade</t>
+        </is>
+      </c>
+      <c r="K313" t="n">
+        <v>12</v>
+      </c>
+      <c r="L313" t="n">
+        <v>22</v>
+      </c>
+      <c r="M313" t="n">
+        <v>0</v>
+      </c>
+      <c r="N313" t="inlineStr">
+        <is>
+          <t>Quick Claw</t>
+        </is>
+      </c>
+      <c r="O313" t="inlineStr">
+        <is>
+          <t>Às vezes age primeiro.</t>
         </is>
       </c>
     </row>
@@ -22655,7 +24143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1325"/>
+  <dimension ref="A1:H1325"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -22703,6 +24191,11 @@
           <t>Categoria da padrão</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Habilidade 3</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -23158,6 +24651,11 @@
           <t>Defesa</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Lum Protection</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -23188,6 +24686,11 @@
           <t>Sem efeito</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Endeavor</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -23343,6 +24846,11 @@
           <t>Static</t>
         </is>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Endeavor</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>Lightning Rod</t>
@@ -23351,6 +24859,11 @@
       <c r="G26" t="inlineStr">
         <is>
           <t>Controle</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Air Balloon</t>
         </is>
       </c>
     </row>
@@ -23638,6 +25151,11 @@
           <t>Controle</t>
         </is>
       </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Air Balloon</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -23748,6 +25266,11 @@
           <t>Controle</t>
         </is>
       </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Air Balloon</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -23793,6 +25316,11 @@
           <t>Inner Focus</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Lum Protection</t>
+        </is>
+      </c>
       <c r="F42" t="inlineStr">
         <is>
           <t>Infiltrator</t>
@@ -25948,6 +27476,11 @@
           <t>Sem efeito</t>
         </is>
       </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>Endeavor</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -26423,6 +27956,11 @@
           <t>Limber</t>
         </is>
       </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>Transform</t>
+        </is>
+      </c>
       <c r="F133" t="inlineStr">
         <is>
           <t>Imposter</t>
@@ -26463,6 +28001,11 @@
           <t>Sem efeito</t>
         </is>
       </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Air Balloon</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -26938,6 +28481,11 @@
           <t>Synchronize</t>
         </is>
       </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Transform</t>
+        </is>
+      </c>
       <c r="G152" t="inlineStr">
         <is>
           <t>Defesa</t>
@@ -28683,6 +30231,11 @@
           <t>Sobrevivência</t>
         </is>
       </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>Air Balloon</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="n">
@@ -29693,6 +31246,11 @@
           <t>Pressure</t>
         </is>
       </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Lum Protection</t>
+        </is>
+      </c>
       <c r="F250" t="inlineStr">
         <is>
           <t>Multiscale</t>
@@ -29813,6 +31371,11 @@
           <t>Overgrow</t>
         </is>
       </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>Endeavor</t>
+        </is>
+      </c>
       <c r="F255" t="inlineStr">
         <is>
           <t>Unburden</t>
@@ -30403,6 +31966,11 @@
           <t>Guts</t>
         </is>
       </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>Endeavor</t>
+        </is>
+      </c>
       <c r="F277" t="inlineStr">
         <is>
           <t>Scrappy</t>
@@ -31173,6 +32741,11 @@
           <t>Sobrevivência</t>
         </is>
       </c>
+      <c r="H305" t="inlineStr">
+        <is>
+          <t>Endeavor</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" t="n">
@@ -32533,6 +34106,11 @@
           <t>Levitate</t>
         </is>
       </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>Wonder Room</t>
+        </is>
+      </c>
       <c r="F356" t="inlineStr">
         <is>
           <t>Frisk</t>
@@ -33608,6 +35186,11 @@
           <t>Intimidate</t>
         </is>
       </c>
+      <c r="E399" t="inlineStr">
+        <is>
+          <t>Lum Protection</t>
+        </is>
+      </c>
       <c r="F399" t="inlineStr">
         <is>
           <t>Reckless</t>
@@ -34343,6 +35926,11 @@
           <t>Reflexo</t>
         </is>
       </c>
+      <c r="H426" t="inlineStr">
+        <is>
+          <t>Air Balloon</t>
+        </is>
+      </c>
     </row>
     <row r="427">
       <c r="A427" t="n">
@@ -34653,6 +36241,11 @@
           <t>Defesa</t>
         </is>
       </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>Wonder Room</t>
+        </is>
+      </c>
     </row>
     <row r="438">
       <c r="A438" t="n">
@@ -35548,6 +37141,11 @@
           <t>Dano</t>
         </is>
       </c>
+      <c r="H469" t="inlineStr">
+        <is>
+          <t>Lum Protection</t>
+        </is>
+      </c>
     </row>
     <row r="470">
       <c r="A470" t="n">
@@ -35688,6 +37286,11 @@
           <t>Defesa</t>
         </is>
       </c>
+      <c r="H474" t="inlineStr">
+        <is>
+          <t>Endeavor</t>
+        </is>
+      </c>
     </row>
     <row r="475">
       <c r="A475" t="n">
@@ -35863,6 +37466,11 @@
           <t>Levitate</t>
         </is>
       </c>
+      <c r="E481" t="inlineStr">
+        <is>
+          <t>Wonder Room</t>
+        </is>
+      </c>
       <c r="G481" t="inlineStr">
         <is>
           <t>Defesa</t>
@@ -36903,6 +38511,11 @@
           <t>Defesa</t>
         </is>
       </c>
+      <c r="H522" t="inlineStr">
+        <is>
+          <t>Lum Protection</t>
+        </is>
+      </c>
     </row>
     <row r="523">
       <c r="A523" t="n">
@@ -38363,6 +39976,11 @@
           <t>Controle</t>
         </is>
       </c>
+      <c r="H573" t="inlineStr">
+        <is>
+          <t>Air Balloon</t>
+        </is>
+      </c>
     </row>
     <row r="574">
       <c r="A574" t="n">
@@ -38798,6 +40416,11 @@
           <t>Static</t>
         </is>
       </c>
+      <c r="E588" t="inlineStr">
+        <is>
+          <t>Air Balloon</t>
+        </is>
+      </c>
       <c r="F588" t="inlineStr">
         <is>
           <t>Motor Drive</t>
@@ -40808,6 +42431,11 @@
           <t>Flame Body</t>
         </is>
       </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>Lum Protection</t>
+        </is>
+      </c>
       <c r="F664" t="inlineStr">
         <is>
           <t>Gale Wings</t>
@@ -42233,6 +43861,11 @@
           <t>Sem efeito</t>
         </is>
       </c>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>Lum Protection</t>
+        </is>
+      </c>
     </row>
     <row r="717">
       <c r="A717" t="n">
@@ -42328,6 +43961,11 @@
           <t>Magician</t>
         </is>
       </c>
+      <c r="E721" t="inlineStr">
+        <is>
+          <t>Wonder Room</t>
+        </is>
+      </c>
       <c r="G721" t="inlineStr">
         <is>
           <t>Sem efeito</t>
@@ -42668,6 +44306,11 @@
           <t>Defesa</t>
         </is>
       </c>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>Lum Protection</t>
+        </is>
+      </c>
     </row>
     <row r="735">
       <c r="A735" t="n">
@@ -45893,6 +47536,11 @@
           <t>Suporte</t>
         </is>
       </c>
+      <c r="H859" t="inlineStr">
+        <is>
+          <t>Wonder Room</t>
+        </is>
+      </c>
     </row>
     <row r="860">
       <c r="A860" t="n">
@@ -46181,6 +47829,11 @@
       <c r="D870" t="inlineStr">
         <is>
           <t>Sweet Veil</t>
+        </is>
+      </c>
+      <c r="E870" t="inlineStr">
+        <is>
+          <t>Wonder Room</t>
         </is>
       </c>
       <c r="F870" t="inlineStr">

</xml_diff>